<commit_message>
otro fix de plantilla variador
</commit_message>
<xml_diff>
--- a/public/informes-templates/INFORME VARIADOR REPARACION.xlsx
+++ b/public/informes-templates/INFORME VARIADOR REPARACION.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30326"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9DE03762-3C24-462B-8368-DD60F0A5B27C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{02C4A046-F2A7-472F-A6F8-996D3E80A366}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -359,7 +359,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="17">
+  <borders count="20">
     <border>
       <left/>
       <right/>
@@ -551,11 +551,48 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="84">
+  <cellXfs count="80">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -602,20 +639,44 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="49" fontId="5" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
@@ -623,8 +684,41 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="12" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
@@ -632,25 +726,28 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="5" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="9" fillId="3" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -659,65 +756,26 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="9" fillId="3" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="5" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="12" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -752,58 +810,27 @@
     <xf numFmtId="0" fontId="6" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="4" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="49" fontId="5" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="4" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1022,24 +1049,24 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:Z350"/>
+  <dimension ref="A1:Z349"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="14.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="9" width="18.85546875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:26" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="20" t="s">
+      <c r="A1" s="73" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="21"/>
-      <c r="C1" s="21"/>
-      <c r="D1" s="21"/>
-      <c r="E1" s="21"/>
-      <c r="F1" s="21"/>
-      <c r="G1" s="21"/>
-      <c r="H1" s="21"/>
-      <c r="I1" s="22"/>
+      <c r="B1" s="29"/>
+      <c r="C1" s="29"/>
+      <c r="D1" s="29"/>
+      <c r="E1" s="29"/>
+      <c r="F1" s="29"/>
+      <c r="G1" s="29"/>
+      <c r="H1" s="29"/>
+      <c r="I1" s="30"/>
       <c r="J1" s="1"/>
       <c r="K1" s="1"/>
       <c r="L1" s="1"/>
@@ -1059,15 +1086,15 @@
       <c r="Z1" s="1"/>
     </row>
     <row r="2" spans="1:26" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="23"/>
-      <c r="B2" s="24"/>
-      <c r="C2" s="24"/>
-      <c r="D2" s="24"/>
-      <c r="E2" s="24"/>
-      <c r="F2" s="24"/>
-      <c r="G2" s="24"/>
-      <c r="H2" s="24"/>
-      <c r="I2" s="25"/>
+      <c r="A2" s="58"/>
+      <c r="B2" s="43"/>
+      <c r="C2" s="43"/>
+      <c r="D2" s="43"/>
+      <c r="E2" s="43"/>
+      <c r="F2" s="43"/>
+      <c r="G2" s="43"/>
+      <c r="H2" s="43"/>
+      <c r="I2" s="44"/>
       <c r="J2" s="1"/>
       <c r="K2" s="1"/>
       <c r="L2" s="1"/>
@@ -1087,15 +1114,15 @@
       <c r="Z2" s="1"/>
     </row>
     <row r="3" spans="1:26" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="52"/>
-      <c r="B3" s="53"/>
-      <c r="C3" s="53"/>
-      <c r="D3" s="53"/>
-      <c r="E3" s="53"/>
-      <c r="F3" s="53"/>
-      <c r="G3" s="53"/>
-      <c r="H3" s="53"/>
-      <c r="I3" s="54"/>
+      <c r="A3" s="74"/>
+      <c r="B3" s="75"/>
+      <c r="C3" s="75"/>
+      <c r="D3" s="75"/>
+      <c r="E3" s="75"/>
+      <c r="F3" s="75"/>
+      <c r="G3" s="75"/>
+      <c r="H3" s="75"/>
+      <c r="I3" s="76"/>
       <c r="J3" s="1"/>
       <c r="K3" s="1"/>
       <c r="L3" s="1"/>
@@ -1115,15 +1142,15 @@
       <c r="Z3" s="1"/>
     </row>
     <row r="4" spans="1:26" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="27"/>
-      <c r="B4" s="24"/>
-      <c r="C4" s="24"/>
-      <c r="D4" s="24"/>
-      <c r="E4" s="24"/>
-      <c r="F4" s="24"/>
-      <c r="G4" s="24"/>
-      <c r="H4" s="24"/>
-      <c r="I4" s="24"/>
+      <c r="A4" s="60"/>
+      <c r="B4" s="43"/>
+      <c r="C4" s="43"/>
+      <c r="D4" s="43"/>
+      <c r="E4" s="43"/>
+      <c r="F4" s="43"/>
+      <c r="G4" s="43"/>
+      <c r="H4" s="43"/>
+      <c r="I4" s="43"/>
       <c r="J4" s="1"/>
       <c r="K4" s="1"/>
       <c r="L4" s="1"/>
@@ -1143,17 +1170,17 @@
       <c r="Z4" s="1"/>
     </row>
     <row r="5" spans="1:26" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="36" t="s">
+      <c r="A5" s="57" t="s">
         <v>2</v>
       </c>
-      <c r="B5" s="55"/>
-      <c r="C5" s="55"/>
-      <c r="D5" s="55"/>
-      <c r="E5" s="55"/>
-      <c r="F5" s="55"/>
-      <c r="G5" s="55"/>
-      <c r="H5" s="55"/>
-      <c r="I5" s="56"/>
+      <c r="B5" s="62"/>
+      <c r="C5" s="62"/>
+      <c r="D5" s="62"/>
+      <c r="E5" s="62"/>
+      <c r="F5" s="62"/>
+      <c r="G5" s="62"/>
+      <c r="H5" s="62"/>
+      <c r="I5" s="63"/>
       <c r="J5" s="1"/>
       <c r="K5" s="1"/>
       <c r="L5" s="1"/>
@@ -1173,18 +1200,18 @@
       <c r="Z5" s="1"/>
     </row>
     <row r="6" spans="1:26" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="57" t="s">
+      <c r="A6" s="64" t="s">
         <v>3</v>
       </c>
-      <c r="B6" s="58"/>
-      <c r="C6" s="57" t="s">
+      <c r="B6" s="65"/>
+      <c r="C6" s="64" t="s">
         <v>4</v>
       </c>
-      <c r="D6" s="58"/>
-      <c r="E6" s="28" t="s">
+      <c r="D6" s="65"/>
+      <c r="E6" s="35" t="s">
         <v>5</v>
       </c>
-      <c r="F6" s="30"/>
+      <c r="F6" s="34"/>
       <c r="G6" s="3" t="s">
         <v>6</v>
       </c>
@@ -1213,15 +1240,15 @@
       <c r="Z6" s="1"/>
     </row>
     <row r="7" spans="1:26" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="61"/>
-      <c r="B7" s="62"/>
-      <c r="C7" s="59"/>
-      <c r="D7" s="60"/>
-      <c r="E7" s="66"/>
-      <c r="F7" s="22"/>
-      <c r="G7" s="19"/>
-      <c r="H7" s="19"/>
-      <c r="I7" s="19"/>
+      <c r="A7" s="68"/>
+      <c r="B7" s="69"/>
+      <c r="C7" s="66"/>
+      <c r="D7" s="67"/>
+      <c r="E7" s="61"/>
+      <c r="F7" s="30"/>
+      <c r="G7" s="16"/>
+      <c r="H7" s="16"/>
+      <c r="I7" s="16"/>
       <c r="J7" s="1"/>
       <c r="K7" s="1"/>
       <c r="L7" s="1"/>
@@ -1241,19 +1268,19 @@
       <c r="Z7" s="1"/>
     </row>
     <row r="8" spans="1:26" x14ac:dyDescent="0.25">
-      <c r="A8" s="57" t="s">
+      <c r="A8" s="64" t="s">
         <v>9</v>
       </c>
-      <c r="B8" s="58"/>
-      <c r="C8" s="36" t="s">
+      <c r="B8" s="65"/>
+      <c r="C8" s="57" t="s">
         <v>10</v>
       </c>
-      <c r="D8" s="69"/>
-      <c r="E8" s="69"/>
-      <c r="F8" s="69"/>
-      <c r="G8" s="69"/>
-      <c r="H8" s="69"/>
-      <c r="I8" s="69"/>
+      <c r="D8" s="27"/>
+      <c r="E8" s="27"/>
+      <c r="F8" s="27"/>
+      <c r="G8" s="27"/>
+      <c r="H8" s="27"/>
+      <c r="I8" s="27"/>
       <c r="J8" s="1"/>
       <c r="K8" s="1"/>
       <c r="L8" s="1"/>
@@ -1273,15 +1300,15 @@
       <c r="Z8" s="1"/>
     </row>
     <row r="9" spans="1:26" x14ac:dyDescent="0.25">
-      <c r="A9" s="63"/>
-      <c r="B9" s="64"/>
-      <c r="C9" s="65"/>
-      <c r="D9" s="69"/>
-      <c r="E9" s="69"/>
-      <c r="F9" s="69"/>
-      <c r="G9" s="69"/>
-      <c r="H9" s="69"/>
-      <c r="I9" s="69"/>
+      <c r="A9" s="70"/>
+      <c r="B9" s="71"/>
+      <c r="C9" s="72"/>
+      <c r="D9" s="27"/>
+      <c r="E9" s="27"/>
+      <c r="F9" s="27"/>
+      <c r="G9" s="27"/>
+      <c r="H9" s="27"/>
+      <c r="I9" s="27"/>
       <c r="J9" s="1"/>
       <c r="K9" s="1"/>
       <c r="L9" s="1"/>
@@ -1301,19 +1328,19 @@
       <c r="Z9" s="1"/>
     </row>
     <row r="10" spans="1:26" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="32" t="s">
+      <c r="A10" s="31" t="s">
         <v>11</v>
       </c>
-      <c r="B10" s="21"/>
-      <c r="C10" s="21"/>
-      <c r="D10" s="67"/>
+      <c r="B10" s="29"/>
+      <c r="C10" s="29"/>
+      <c r="D10" s="51"/>
       <c r="E10" s="5"/>
-      <c r="F10" s="68" t="s">
+      <c r="F10" s="52" t="s">
         <v>12</v>
       </c>
-      <c r="G10" s="67"/>
-      <c r="H10" s="67"/>
-      <c r="I10" s="67"/>
+      <c r="G10" s="51"/>
+      <c r="H10" s="51"/>
+      <c r="I10" s="51"/>
       <c r="J10" s="1"/>
       <c r="K10" s="1"/>
       <c r="L10" s="1"/>
@@ -1339,7 +1366,7 @@
       <c r="B11" s="6"/>
       <c r="C11" s="10"/>
       <c r="D11" s="11"/>
-      <c r="E11" s="33"/>
+      <c r="E11" s="53"/>
       <c r="F11" s="2" t="s">
         <v>13</v>
       </c>
@@ -1371,7 +1398,7 @@
       <c r="B12" s="6"/>
       <c r="C12" s="12"/>
       <c r="D12" s="13"/>
-      <c r="E12" s="34"/>
+      <c r="E12" s="54"/>
       <c r="F12" s="2" t="s">
         <v>14</v>
       </c>
@@ -1403,7 +1430,7 @@
       <c r="B13" s="6"/>
       <c r="C13" s="12"/>
       <c r="D13" s="13"/>
-      <c r="E13" s="34"/>
+      <c r="E13" s="54"/>
       <c r="F13" s="2" t="s">
         <v>15</v>
       </c>
@@ -1435,7 +1462,7 @@
       <c r="B14" s="4"/>
       <c r="C14" s="12"/>
       <c r="D14" s="13"/>
-      <c r="E14" s="34"/>
+      <c r="E14" s="54"/>
       <c r="F14" s="2" t="s">
         <v>16</v>
       </c>
@@ -1467,7 +1494,7 @@
       <c r="B15" s="6"/>
       <c r="C15" s="12"/>
       <c r="D15" s="13"/>
-      <c r="E15" s="34"/>
+      <c r="E15" s="54"/>
       <c r="F15" s="2" t="s">
         <v>17</v>
       </c>
@@ -1499,7 +1526,7 @@
       <c r="B16" s="4"/>
       <c r="C16" s="12"/>
       <c r="D16" s="13"/>
-      <c r="E16" s="34"/>
+      <c r="E16" s="54"/>
       <c r="F16" s="2" t="s">
         <v>18</v>
       </c>
@@ -1531,7 +1558,7 @@
       <c r="B17" s="4"/>
       <c r="C17" s="12"/>
       <c r="D17" s="13"/>
-      <c r="E17" s="34"/>
+      <c r="E17" s="54"/>
       <c r="F17" s="2" t="s">
         <v>19</v>
       </c>
@@ -1563,7 +1590,7 @@
       <c r="B18" s="4"/>
       <c r="C18" s="12"/>
       <c r="D18" s="13"/>
-      <c r="E18" s="34"/>
+      <c r="E18" s="54"/>
       <c r="F18" s="2" t="s">
         <v>20</v>
       </c>
@@ -1595,7 +1622,7 @@
       <c r="B19" s="4"/>
       <c r="C19" s="12"/>
       <c r="D19" s="13"/>
-      <c r="E19" s="34"/>
+      <c r="E19" s="54"/>
       <c r="F19" s="2" t="s">
         <v>21</v>
       </c>
@@ -1627,7 +1654,7 @@
       <c r="B20" s="4"/>
       <c r="C20" s="12"/>
       <c r="D20" s="13"/>
-      <c r="E20" s="34"/>
+      <c r="E20" s="54"/>
       <c r="F20" s="2" t="s">
         <v>22</v>
       </c>
@@ -1659,7 +1686,7 @@
       <c r="B21" s="4"/>
       <c r="C21" s="12"/>
       <c r="D21" s="13"/>
-      <c r="E21" s="34"/>
+      <c r="E21" s="54"/>
       <c r="F21" s="2" t="s">
         <v>23</v>
       </c>
@@ -1691,7 +1718,7 @@
       <c r="B22" s="4"/>
       <c r="C22" s="12"/>
       <c r="D22" s="13"/>
-      <c r="E22" s="34"/>
+      <c r="E22" s="54"/>
       <c r="F22" s="2" t="s">
         <v>24</v>
       </c>
@@ -1723,7 +1750,7 @@
       <c r="B23" s="4"/>
       <c r="C23" s="14"/>
       <c r="D23" s="15"/>
-      <c r="E23" s="34"/>
+      <c r="E23" s="54"/>
       <c r="F23" s="2" t="s">
         <v>25</v>
       </c>
@@ -1749,23 +1776,23 @@
       <c r="Z23" s="1"/>
     </row>
     <row r="24" spans="1:26" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="35" t="s">
+      <c r="A24" s="56" t="s">
         <v>26</v>
       </c>
-      <c r="B24" s="30"/>
-      <c r="C24" s="36" t="s">
+      <c r="B24" s="34"/>
+      <c r="C24" s="57" t="s">
         <v>27</v>
       </c>
-      <c r="D24" s="22"/>
-      <c r="E24" s="34"/>
-      <c r="F24" s="35" t="s">
+      <c r="D24" s="30"/>
+      <c r="E24" s="54"/>
+      <c r="F24" s="56" t="s">
         <v>26</v>
       </c>
-      <c r="G24" s="30"/>
-      <c r="H24" s="36" t="s">
+      <c r="G24" s="34"/>
+      <c r="H24" s="57" t="s">
         <v>28</v>
       </c>
-      <c r="I24" s="22"/>
+      <c r="I24" s="30"/>
       <c r="J24" s="1"/>
       <c r="K24" s="1"/>
       <c r="L24" s="1"/>
@@ -1785,15 +1812,15 @@
       <c r="Z24" s="1"/>
     </row>
     <row r="25" spans="1:26" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="37"/>
-      <c r="B25" s="25"/>
-      <c r="C25" s="23"/>
-      <c r="D25" s="25"/>
-      <c r="E25" s="31"/>
-      <c r="F25" s="37"/>
-      <c r="G25" s="25"/>
-      <c r="H25" s="23"/>
-      <c r="I25" s="25"/>
+      <c r="A25" s="59"/>
+      <c r="B25" s="44"/>
+      <c r="C25" s="58"/>
+      <c r="D25" s="44"/>
+      <c r="E25" s="55"/>
+      <c r="F25" s="59"/>
+      <c r="G25" s="44"/>
+      <c r="H25" s="58"/>
+      <c r="I25" s="44"/>
       <c r="J25" s="1"/>
       <c r="K25" s="1"/>
       <c r="L25" s="1"/>
@@ -1813,17 +1840,17 @@
       <c r="Z25" s="1"/>
     </row>
     <row r="26" spans="1:26" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="40" t="s">
+      <c r="A26" s="50" t="s">
         <v>29</v>
       </c>
-      <c r="B26" s="29"/>
-      <c r="C26" s="29"/>
-      <c r="D26" s="29"/>
-      <c r="E26" s="29"/>
-      <c r="F26" s="29"/>
-      <c r="G26" s="29"/>
-      <c r="H26" s="29"/>
-      <c r="I26" s="30"/>
+      <c r="B26" s="33"/>
+      <c r="C26" s="33"/>
+      <c r="D26" s="33"/>
+      <c r="E26" s="33"/>
+      <c r="F26" s="33"/>
+      <c r="G26" s="33"/>
+      <c r="H26" s="33"/>
+      <c r="I26" s="34"/>
       <c r="J26" s="1"/>
       <c r="K26" s="1"/>
       <c r="L26" s="1"/>
@@ -1843,15 +1870,15 @@
       <c r="Z26" s="1"/>
     </row>
     <row r="27" spans="1:26" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="70"/>
-      <c r="B27" s="71"/>
-      <c r="C27" s="72"/>
-      <c r="D27" s="70"/>
-      <c r="E27" s="71"/>
-      <c r="F27" s="72"/>
-      <c r="G27" s="70"/>
-      <c r="H27" s="71"/>
-      <c r="I27" s="72"/>
+      <c r="A27" s="17"/>
+      <c r="B27" s="18"/>
+      <c r="C27" s="19"/>
+      <c r="D27" s="17"/>
+      <c r="E27" s="18"/>
+      <c r="F27" s="19"/>
+      <c r="G27" s="17"/>
+      <c r="H27" s="18"/>
+      <c r="I27" s="19"/>
       <c r="J27" s="1"/>
       <c r="K27" s="1"/>
       <c r="L27" s="1"/>
@@ -1871,15 +1898,15 @@
       <c r="Z27" s="1"/>
     </row>
     <row r="28" spans="1:26" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A28" s="73"/>
-      <c r="B28" s="74"/>
-      <c r="C28" s="75"/>
-      <c r="D28" s="73"/>
-      <c r="E28" s="74"/>
-      <c r="F28" s="75"/>
-      <c r="G28" s="73"/>
-      <c r="H28" s="74"/>
-      <c r="I28" s="75"/>
+      <c r="A28" s="20"/>
+      <c r="B28" s="21"/>
+      <c r="C28" s="22"/>
+      <c r="D28" s="20"/>
+      <c r="E28" s="21"/>
+      <c r="F28" s="22"/>
+      <c r="G28" s="20"/>
+      <c r="H28" s="21"/>
+      <c r="I28" s="22"/>
       <c r="J28" s="1"/>
       <c r="K28" s="1"/>
       <c r="L28" s="1"/>
@@ -1899,15 +1926,15 @@
       <c r="Z28" s="1"/>
     </row>
     <row r="29" spans="1:26" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="73"/>
-      <c r="B29" s="74"/>
-      <c r="C29" s="75"/>
-      <c r="D29" s="73"/>
-      <c r="E29" s="74"/>
-      <c r="F29" s="75"/>
-      <c r="G29" s="73"/>
-      <c r="H29" s="74"/>
-      <c r="I29" s="75"/>
+      <c r="A29" s="20"/>
+      <c r="B29" s="21"/>
+      <c r="C29" s="22"/>
+      <c r="D29" s="20"/>
+      <c r="E29" s="21"/>
+      <c r="F29" s="22"/>
+      <c r="G29" s="20"/>
+      <c r="H29" s="21"/>
+      <c r="I29" s="22"/>
       <c r="J29" s="1"/>
       <c r="K29" s="1"/>
       <c r="L29" s="1"/>
@@ -1927,15 +1954,15 @@
       <c r="Z29" s="1"/>
     </row>
     <row r="30" spans="1:26" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A30" s="73"/>
-      <c r="B30" s="74"/>
-      <c r="C30" s="75"/>
-      <c r="D30" s="73"/>
-      <c r="E30" s="74"/>
-      <c r="F30" s="75"/>
-      <c r="G30" s="73"/>
-      <c r="H30" s="74"/>
-      <c r="I30" s="75"/>
+      <c r="A30" s="20"/>
+      <c r="B30" s="21"/>
+      <c r="C30" s="22"/>
+      <c r="D30" s="20"/>
+      <c r="E30" s="21"/>
+      <c r="F30" s="22"/>
+      <c r="G30" s="20"/>
+      <c r="H30" s="21"/>
+      <c r="I30" s="22"/>
       <c r="J30" s="1"/>
       <c r="K30" s="1"/>
       <c r="L30" s="1"/>
@@ -1955,15 +1982,15 @@
       <c r="Z30" s="1"/>
     </row>
     <row r="31" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A31" s="73"/>
-      <c r="B31" s="74"/>
-      <c r="C31" s="75"/>
-      <c r="D31" s="73"/>
-      <c r="E31" s="74"/>
-      <c r="F31" s="75"/>
-      <c r="G31" s="73"/>
-      <c r="H31" s="74"/>
-      <c r="I31" s="75"/>
+      <c r="A31" s="20"/>
+      <c r="B31" s="21"/>
+      <c r="C31" s="22"/>
+      <c r="D31" s="20"/>
+      <c r="E31" s="21"/>
+      <c r="F31" s="22"/>
+      <c r="G31" s="20"/>
+      <c r="H31" s="21"/>
+      <c r="I31" s="22"/>
       <c r="J31" s="1"/>
       <c r="K31" s="1"/>
       <c r="L31" s="1"/>
@@ -1983,15 +2010,15 @@
       <c r="Z31" s="1"/>
     </row>
     <row r="32" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A32" s="73"/>
-      <c r="B32" s="74"/>
-      <c r="C32" s="75"/>
-      <c r="D32" s="73"/>
-      <c r="E32" s="74"/>
-      <c r="F32" s="75"/>
-      <c r="G32" s="73"/>
-      <c r="H32" s="74"/>
-      <c r="I32" s="75"/>
+      <c r="A32" s="20"/>
+      <c r="B32" s="21"/>
+      <c r="C32" s="22"/>
+      <c r="D32" s="20"/>
+      <c r="E32" s="21"/>
+      <c r="F32" s="22"/>
+      <c r="G32" s="20"/>
+      <c r="H32" s="21"/>
+      <c r="I32" s="22"/>
       <c r="J32" s="1"/>
       <c r="K32" s="1"/>
       <c r="L32" s="1"/>
@@ -2011,15 +2038,15 @@
       <c r="Z32" s="1"/>
     </row>
     <row r="33" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A33" s="73"/>
-      <c r="B33" s="74"/>
-      <c r="C33" s="75"/>
-      <c r="D33" s="73"/>
-      <c r="E33" s="74"/>
-      <c r="F33" s="75"/>
-      <c r="G33" s="73"/>
-      <c r="H33" s="74"/>
-      <c r="I33" s="75"/>
+      <c r="A33" s="20"/>
+      <c r="B33" s="21"/>
+      <c r="C33" s="22"/>
+      <c r="D33" s="20"/>
+      <c r="E33" s="21"/>
+      <c r="F33" s="22"/>
+      <c r="G33" s="20"/>
+      <c r="H33" s="21"/>
+      <c r="I33" s="22"/>
       <c r="J33" s="1"/>
       <c r="K33" s="1"/>
       <c r="L33" s="1"/>
@@ -2039,15 +2066,15 @@
       <c r="Z33" s="1"/>
     </row>
     <row r="34" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A34" s="73"/>
-      <c r="B34" s="74"/>
-      <c r="C34" s="75"/>
-      <c r="D34" s="73"/>
-      <c r="E34" s="74"/>
-      <c r="F34" s="75"/>
-      <c r="G34" s="73"/>
-      <c r="H34" s="74"/>
-      <c r="I34" s="75"/>
+      <c r="A34" s="20"/>
+      <c r="B34" s="21"/>
+      <c r="C34" s="22"/>
+      <c r="D34" s="20"/>
+      <c r="E34" s="21"/>
+      <c r="F34" s="22"/>
+      <c r="G34" s="20"/>
+      <c r="H34" s="21"/>
+      <c r="I34" s="22"/>
       <c r="J34" s="1"/>
       <c r="K34" s="1"/>
       <c r="L34" s="1"/>
@@ -2067,15 +2094,15 @@
       <c r="Z34" s="1"/>
     </row>
     <row r="35" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A35" s="73"/>
-      <c r="B35" s="74"/>
-      <c r="C35" s="75"/>
-      <c r="D35" s="73"/>
-      <c r="E35" s="74"/>
-      <c r="F35" s="75"/>
-      <c r="G35" s="73"/>
-      <c r="H35" s="74"/>
-      <c r="I35" s="75"/>
+      <c r="A35" s="20"/>
+      <c r="B35" s="21"/>
+      <c r="C35" s="22"/>
+      <c r="D35" s="20"/>
+      <c r="E35" s="21"/>
+      <c r="F35" s="22"/>
+      <c r="G35" s="20"/>
+      <c r="H35" s="21"/>
+      <c r="I35" s="22"/>
       <c r="J35" s="1"/>
       <c r="K35" s="1"/>
       <c r="L35" s="1"/>
@@ -2095,15 +2122,15 @@
       <c r="Z35" s="1"/>
     </row>
     <row r="36" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A36" s="73"/>
-      <c r="B36" s="74"/>
-      <c r="C36" s="75"/>
-      <c r="D36" s="73"/>
-      <c r="E36" s="74"/>
-      <c r="F36" s="75"/>
-      <c r="G36" s="73"/>
-      <c r="H36" s="74"/>
-      <c r="I36" s="75"/>
+      <c r="A36" s="20"/>
+      <c r="B36" s="21"/>
+      <c r="C36" s="22"/>
+      <c r="D36" s="20"/>
+      <c r="E36" s="21"/>
+      <c r="F36" s="22"/>
+      <c r="G36" s="20"/>
+      <c r="H36" s="21"/>
+      <c r="I36" s="22"/>
       <c r="J36" s="1"/>
       <c r="K36" s="1"/>
       <c r="L36" s="1"/>
@@ -2123,15 +2150,15 @@
       <c r="Z36" s="1"/>
     </row>
     <row r="37" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A37" s="73"/>
-      <c r="B37" s="74"/>
-      <c r="C37" s="75"/>
-      <c r="D37" s="73"/>
-      <c r="E37" s="74"/>
-      <c r="F37" s="75"/>
-      <c r="G37" s="73"/>
-      <c r="H37" s="74"/>
-      <c r="I37" s="75"/>
+      <c r="A37" s="20"/>
+      <c r="B37" s="21"/>
+      <c r="C37" s="22"/>
+      <c r="D37" s="20"/>
+      <c r="E37" s="21"/>
+      <c r="F37" s="22"/>
+      <c r="G37" s="20"/>
+      <c r="H37" s="21"/>
+      <c r="I37" s="22"/>
       <c r="J37" s="1"/>
       <c r="K37" s="1"/>
       <c r="L37" s="1"/>
@@ -2151,15 +2178,15 @@
       <c r="Z37" s="1"/>
     </row>
     <row r="38" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A38" s="73"/>
-      <c r="B38" s="74"/>
-      <c r="C38" s="75"/>
-      <c r="D38" s="73"/>
-      <c r="E38" s="74"/>
-      <c r="F38" s="75"/>
-      <c r="G38" s="73"/>
-      <c r="H38" s="74"/>
-      <c r="I38" s="75"/>
+      <c r="A38" s="20"/>
+      <c r="B38" s="21"/>
+      <c r="C38" s="22"/>
+      <c r="D38" s="20"/>
+      <c r="E38" s="21"/>
+      <c r="F38" s="22"/>
+      <c r="G38" s="20"/>
+      <c r="H38" s="21"/>
+      <c r="I38" s="22"/>
       <c r="J38" s="1"/>
       <c r="K38" s="1"/>
       <c r="L38" s="1"/>
@@ -2179,15 +2206,15 @@
       <c r="Z38" s="1"/>
     </row>
     <row r="39" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A39" s="73"/>
-      <c r="B39" s="74"/>
-      <c r="C39" s="75"/>
-      <c r="D39" s="73"/>
-      <c r="E39" s="74"/>
-      <c r="F39" s="75"/>
-      <c r="G39" s="73"/>
-      <c r="H39" s="74"/>
-      <c r="I39" s="75"/>
+      <c r="A39" s="20"/>
+      <c r="B39" s="21"/>
+      <c r="C39" s="22"/>
+      <c r="D39" s="20"/>
+      <c r="E39" s="21"/>
+      <c r="F39" s="22"/>
+      <c r="G39" s="20"/>
+      <c r="H39" s="21"/>
+      <c r="I39" s="22"/>
       <c r="J39" s="1"/>
       <c r="K39" s="1"/>
       <c r="L39" s="1"/>
@@ -2207,15 +2234,15 @@
       <c r="Z39" s="1"/>
     </row>
     <row r="40" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A40" s="73"/>
-      <c r="B40" s="74"/>
-      <c r="C40" s="75"/>
-      <c r="D40" s="73"/>
-      <c r="E40" s="74"/>
-      <c r="F40" s="75"/>
-      <c r="G40" s="73"/>
-      <c r="H40" s="74"/>
-      <c r="I40" s="75"/>
+      <c r="A40" s="20"/>
+      <c r="B40" s="21"/>
+      <c r="C40" s="22"/>
+      <c r="D40" s="20"/>
+      <c r="E40" s="21"/>
+      <c r="F40" s="22"/>
+      <c r="G40" s="20"/>
+      <c r="H40" s="21"/>
+      <c r="I40" s="22"/>
       <c r="J40" s="1"/>
       <c r="K40" s="1"/>
       <c r="L40" s="1"/>
@@ -2235,15 +2262,15 @@
       <c r="Z40" s="1"/>
     </row>
     <row r="41" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A41" s="73"/>
-      <c r="B41" s="74"/>
-      <c r="C41" s="75"/>
-      <c r="D41" s="73"/>
-      <c r="E41" s="74"/>
-      <c r="F41" s="75"/>
-      <c r="G41" s="73"/>
-      <c r="H41" s="74"/>
-      <c r="I41" s="75"/>
+      <c r="A41" s="20"/>
+      <c r="B41" s="21"/>
+      <c r="C41" s="22"/>
+      <c r="D41" s="20"/>
+      <c r="E41" s="21"/>
+      <c r="F41" s="22"/>
+      <c r="G41" s="20"/>
+      <c r="H41" s="21"/>
+      <c r="I41" s="22"/>
       <c r="J41" s="1"/>
       <c r="K41" s="1"/>
       <c r="L41" s="1"/>
@@ -2263,15 +2290,15 @@
       <c r="Z41" s="1"/>
     </row>
     <row r="42" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A42" s="73"/>
-      <c r="B42" s="74"/>
-      <c r="C42" s="75"/>
-      <c r="D42" s="73"/>
-      <c r="E42" s="74"/>
-      <c r="F42" s="75"/>
-      <c r="G42" s="73"/>
-      <c r="H42" s="74"/>
-      <c r="I42" s="75"/>
+      <c r="A42" s="20"/>
+      <c r="B42" s="21"/>
+      <c r="C42" s="22"/>
+      <c r="D42" s="20"/>
+      <c r="E42" s="21"/>
+      <c r="F42" s="22"/>
+      <c r="G42" s="20"/>
+      <c r="H42" s="21"/>
+      <c r="I42" s="22"/>
       <c r="J42" s="1"/>
       <c r="K42" s="1"/>
       <c r="L42" s="1"/>
@@ -2291,15 +2318,15 @@
       <c r="Z42" s="1"/>
     </row>
     <row r="43" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A43" s="73"/>
-      <c r="B43" s="74"/>
-      <c r="C43" s="75"/>
-      <c r="D43" s="73"/>
-      <c r="E43" s="74"/>
-      <c r="F43" s="75"/>
-      <c r="G43" s="73"/>
-      <c r="H43" s="74"/>
-      <c r="I43" s="75"/>
+      <c r="A43" s="20"/>
+      <c r="B43" s="21"/>
+      <c r="C43" s="22"/>
+      <c r="D43" s="20"/>
+      <c r="E43" s="21"/>
+      <c r="F43" s="22"/>
+      <c r="G43" s="20"/>
+      <c r="H43" s="21"/>
+      <c r="I43" s="22"/>
       <c r="J43" s="1"/>
       <c r="K43" s="1"/>
       <c r="L43" s="1"/>
@@ -2319,15 +2346,15 @@
       <c r="Z43" s="1"/>
     </row>
     <row r="44" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A44" s="73"/>
-      <c r="B44" s="74"/>
-      <c r="C44" s="75"/>
-      <c r="D44" s="73"/>
-      <c r="E44" s="74"/>
-      <c r="F44" s="75"/>
-      <c r="G44" s="73"/>
-      <c r="H44" s="74"/>
-      <c r="I44" s="75"/>
+      <c r="A44" s="20"/>
+      <c r="B44" s="21"/>
+      <c r="C44" s="22"/>
+      <c r="D44" s="20"/>
+      <c r="E44" s="21"/>
+      <c r="F44" s="22"/>
+      <c r="G44" s="20"/>
+      <c r="H44" s="21"/>
+      <c r="I44" s="22"/>
       <c r="J44" s="1"/>
       <c r="K44" s="1"/>
       <c r="L44" s="1"/>
@@ -2347,15 +2374,15 @@
       <c r="Z44" s="1"/>
     </row>
     <row r="45" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A45" s="73"/>
-      <c r="B45" s="74"/>
-      <c r="C45" s="75"/>
-      <c r="D45" s="73"/>
-      <c r="E45" s="74"/>
-      <c r="F45" s="75"/>
-      <c r="G45" s="73"/>
-      <c r="H45" s="74"/>
-      <c r="I45" s="75"/>
+      <c r="A45" s="20"/>
+      <c r="B45" s="21"/>
+      <c r="C45" s="22"/>
+      <c r="D45" s="20"/>
+      <c r="E45" s="21"/>
+      <c r="F45" s="22"/>
+      <c r="G45" s="20"/>
+      <c r="H45" s="21"/>
+      <c r="I45" s="22"/>
       <c r="J45" s="1"/>
       <c r="K45" s="1"/>
       <c r="L45" s="1"/>
@@ -2375,15 +2402,15 @@
       <c r="Z45" s="1"/>
     </row>
     <row r="46" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A46" s="73"/>
-      <c r="B46" s="74"/>
-      <c r="C46" s="75"/>
-      <c r="D46" s="76"/>
-      <c r="E46" s="77"/>
-      <c r="F46" s="78"/>
-      <c r="G46" s="76"/>
-      <c r="H46" s="77"/>
-      <c r="I46" s="78"/>
+      <c r="A46" s="20"/>
+      <c r="B46" s="21"/>
+      <c r="C46" s="22"/>
+      <c r="D46" s="23"/>
+      <c r="E46" s="24"/>
+      <c r="F46" s="25"/>
+      <c r="G46" s="23"/>
+      <c r="H46" s="24"/>
+      <c r="I46" s="25"/>
       <c r="J46" s="1"/>
       <c r="K46" s="1"/>
       <c r="L46" s="1"/>
@@ -2403,21 +2430,21 @@
       <c r="Z46" s="1"/>
     </row>
     <row r="47" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A47" s="38" t="s">
+      <c r="A47" s="40" t="s">
         <v>30</v>
       </c>
-      <c r="B47" s="29"/>
-      <c r="C47" s="30"/>
-      <c r="D47" s="38" t="s">
+      <c r="B47" s="33"/>
+      <c r="C47" s="34"/>
+      <c r="D47" s="40" t="s">
         <v>31</v>
       </c>
-      <c r="E47" s="29"/>
-      <c r="F47" s="30"/>
-      <c r="G47" s="38" t="s">
+      <c r="E47" s="33"/>
+      <c r="F47" s="34"/>
+      <c r="G47" s="40" t="s">
         <v>32</v>
       </c>
-      <c r="H47" s="29"/>
-      <c r="I47" s="30"/>
+      <c r="H47" s="33"/>
+      <c r="I47" s="34"/>
       <c r="J47" s="1"/>
       <c r="K47" s="1"/>
       <c r="L47" s="1"/>
@@ -2437,15 +2464,15 @@
       <c r="Z47" s="1"/>
     </row>
     <row r="48" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A48" s="70"/>
-      <c r="B48" s="71"/>
-      <c r="C48" s="72"/>
-      <c r="D48" s="70"/>
-      <c r="E48" s="71"/>
-      <c r="F48" s="72"/>
-      <c r="G48" s="70"/>
-      <c r="H48" s="71"/>
-      <c r="I48" s="72"/>
+      <c r="A48" s="17"/>
+      <c r="B48" s="18"/>
+      <c r="C48" s="19"/>
+      <c r="D48" s="17"/>
+      <c r="E48" s="18"/>
+      <c r="F48" s="19"/>
+      <c r="G48" s="17"/>
+      <c r="H48" s="18"/>
+      <c r="I48" s="19"/>
       <c r="J48" s="1"/>
       <c r="K48" s="1"/>
       <c r="L48" s="1"/>
@@ -2465,15 +2492,15 @@
       <c r="Z48" s="1"/>
     </row>
     <row r="49" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A49" s="73"/>
-      <c r="B49" s="74"/>
-      <c r="C49" s="75"/>
-      <c r="D49" s="73"/>
-      <c r="E49" s="74"/>
-      <c r="F49" s="75"/>
-      <c r="G49" s="73"/>
-      <c r="H49" s="74"/>
-      <c r="I49" s="75"/>
+      <c r="A49" s="20"/>
+      <c r="B49" s="21"/>
+      <c r="C49" s="22"/>
+      <c r="D49" s="20"/>
+      <c r="E49" s="21"/>
+      <c r="F49" s="22"/>
+      <c r="G49" s="20"/>
+      <c r="H49" s="21"/>
+      <c r="I49" s="22"/>
       <c r="J49" s="1"/>
       <c r="K49" s="1"/>
       <c r="L49" s="1"/>
@@ -2493,15 +2520,15 @@
       <c r="Z49" s="1"/>
     </row>
     <row r="50" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A50" s="73"/>
-      <c r="B50" s="74"/>
-      <c r="C50" s="75"/>
-      <c r="D50" s="73"/>
-      <c r="E50" s="74"/>
-      <c r="F50" s="75"/>
-      <c r="G50" s="73"/>
-      <c r="H50" s="74"/>
-      <c r="I50" s="75"/>
+      <c r="A50" s="20"/>
+      <c r="B50" s="21"/>
+      <c r="C50" s="22"/>
+      <c r="D50" s="20"/>
+      <c r="E50" s="21"/>
+      <c r="F50" s="22"/>
+      <c r="G50" s="20"/>
+      <c r="H50" s="21"/>
+      <c r="I50" s="22"/>
       <c r="J50" s="1"/>
       <c r="K50" s="1"/>
       <c r="L50" s="1"/>
@@ -2521,15 +2548,15 @@
       <c r="Z50" s="1"/>
     </row>
     <row r="51" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A51" s="73"/>
-      <c r="B51" s="74"/>
-      <c r="C51" s="75"/>
-      <c r="D51" s="73"/>
-      <c r="E51" s="74"/>
-      <c r="F51" s="75"/>
-      <c r="G51" s="73"/>
-      <c r="H51" s="74"/>
-      <c r="I51" s="75"/>
+      <c r="A51" s="20"/>
+      <c r="B51" s="21"/>
+      <c r="C51" s="22"/>
+      <c r="D51" s="20"/>
+      <c r="E51" s="21"/>
+      <c r="F51" s="22"/>
+      <c r="G51" s="20"/>
+      <c r="H51" s="21"/>
+      <c r="I51" s="22"/>
       <c r="J51" s="1"/>
       <c r="K51" s="1"/>
       <c r="L51" s="1"/>
@@ -2549,15 +2576,15 @@
       <c r="Z51" s="1"/>
     </row>
     <row r="52" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A52" s="73"/>
-      <c r="B52" s="74"/>
-      <c r="C52" s="75"/>
-      <c r="D52" s="73"/>
-      <c r="E52" s="74"/>
-      <c r="F52" s="75"/>
-      <c r="G52" s="73"/>
-      <c r="H52" s="74"/>
-      <c r="I52" s="75"/>
+      <c r="A52" s="20"/>
+      <c r="B52" s="21"/>
+      <c r="C52" s="22"/>
+      <c r="D52" s="20"/>
+      <c r="E52" s="21"/>
+      <c r="F52" s="22"/>
+      <c r="G52" s="20"/>
+      <c r="H52" s="21"/>
+      <c r="I52" s="22"/>
       <c r="J52" s="1"/>
       <c r="K52" s="1"/>
       <c r="L52" s="1"/>
@@ -2577,15 +2604,15 @@
       <c r="Z52" s="1"/>
     </row>
     <row r="53" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A53" s="73"/>
-      <c r="B53" s="74"/>
-      <c r="C53" s="75"/>
-      <c r="D53" s="73"/>
-      <c r="E53" s="74"/>
-      <c r="F53" s="75"/>
-      <c r="G53" s="73"/>
-      <c r="H53" s="74"/>
-      <c r="I53" s="75"/>
+      <c r="A53" s="20"/>
+      <c r="B53" s="21"/>
+      <c r="C53" s="22"/>
+      <c r="D53" s="20"/>
+      <c r="E53" s="21"/>
+      <c r="F53" s="22"/>
+      <c r="G53" s="20"/>
+      <c r="H53" s="21"/>
+      <c r="I53" s="22"/>
       <c r="J53" s="1"/>
       <c r="K53" s="1"/>
       <c r="L53" s="1"/>
@@ -2605,15 +2632,15 @@
       <c r="Z53" s="1"/>
     </row>
     <row r="54" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A54" s="73"/>
-      <c r="B54" s="74"/>
-      <c r="C54" s="75"/>
-      <c r="D54" s="73"/>
-      <c r="E54" s="74"/>
-      <c r="F54" s="75"/>
-      <c r="G54" s="73"/>
-      <c r="H54" s="74"/>
-      <c r="I54" s="75"/>
+      <c r="A54" s="20"/>
+      <c r="B54" s="21"/>
+      <c r="C54" s="22"/>
+      <c r="D54" s="20"/>
+      <c r="E54" s="21"/>
+      <c r="F54" s="22"/>
+      <c r="G54" s="20"/>
+      <c r="H54" s="21"/>
+      <c r="I54" s="22"/>
       <c r="J54" s="1"/>
       <c r="K54" s="1"/>
       <c r="L54" s="1"/>
@@ -2633,15 +2660,15 @@
       <c r="Z54" s="1"/>
     </row>
     <row r="55" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A55" s="73"/>
-      <c r="B55" s="74"/>
-      <c r="C55" s="75"/>
-      <c r="D55" s="73"/>
-      <c r="E55" s="74"/>
-      <c r="F55" s="75"/>
-      <c r="G55" s="73"/>
-      <c r="H55" s="74"/>
-      <c r="I55" s="75"/>
+      <c r="A55" s="20"/>
+      <c r="B55" s="21"/>
+      <c r="C55" s="22"/>
+      <c r="D55" s="20"/>
+      <c r="E55" s="21"/>
+      <c r="F55" s="22"/>
+      <c r="G55" s="20"/>
+      <c r="H55" s="21"/>
+      <c r="I55" s="22"/>
       <c r="J55" s="1"/>
       <c r="K55" s="1"/>
       <c r="L55" s="1"/>
@@ -2661,15 +2688,15 @@
       <c r="Z55" s="1"/>
     </row>
     <row r="56" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A56" s="73"/>
-      <c r="B56" s="74"/>
-      <c r="C56" s="75"/>
-      <c r="D56" s="73"/>
-      <c r="E56" s="74"/>
-      <c r="F56" s="75"/>
-      <c r="G56" s="73"/>
-      <c r="H56" s="74"/>
-      <c r="I56" s="75"/>
+      <c r="A56" s="20"/>
+      <c r="B56" s="21"/>
+      <c r="C56" s="22"/>
+      <c r="D56" s="20"/>
+      <c r="E56" s="21"/>
+      <c r="F56" s="22"/>
+      <c r="G56" s="20"/>
+      <c r="H56" s="21"/>
+      <c r="I56" s="22"/>
       <c r="J56" s="1"/>
       <c r="K56" s="1"/>
       <c r="L56" s="1"/>
@@ -2689,15 +2716,15 @@
       <c r="Z56" s="1"/>
     </row>
     <row r="57" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A57" s="73"/>
-      <c r="B57" s="74"/>
-      <c r="C57" s="75"/>
-      <c r="D57" s="76"/>
-      <c r="E57" s="77"/>
-      <c r="F57" s="78"/>
-      <c r="G57" s="76"/>
-      <c r="H57" s="77"/>
-      <c r="I57" s="78"/>
+      <c r="A57" s="20"/>
+      <c r="B57" s="21"/>
+      <c r="C57" s="22"/>
+      <c r="D57" s="23"/>
+      <c r="E57" s="24"/>
+      <c r="F57" s="25"/>
+      <c r="G57" s="23"/>
+      <c r="H57" s="24"/>
+      <c r="I57" s="25"/>
       <c r="J57" s="1"/>
       <c r="K57" s="1"/>
       <c r="L57" s="1"/>
@@ -2717,15 +2744,15 @@
       <c r="Z57" s="1"/>
     </row>
     <row r="58" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A58" s="73"/>
-      <c r="B58" s="74"/>
-      <c r="C58" s="75"/>
-      <c r="D58" s="70"/>
-      <c r="E58" s="71"/>
-      <c r="F58" s="72"/>
-      <c r="G58" s="70"/>
-      <c r="H58" s="71"/>
-      <c r="I58" s="72"/>
+      <c r="A58" s="20"/>
+      <c r="B58" s="21"/>
+      <c r="C58" s="22"/>
+      <c r="D58" s="17"/>
+      <c r="E58" s="18"/>
+      <c r="F58" s="19"/>
+      <c r="G58" s="17"/>
+      <c r="H58" s="18"/>
+      <c r="I58" s="19"/>
       <c r="J58" s="1"/>
       <c r="K58" s="1"/>
       <c r="L58" s="1"/>
@@ -2745,15 +2772,15 @@
       <c r="Z58" s="1"/>
     </row>
     <row r="59" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A59" s="73"/>
-      <c r="B59" s="74"/>
-      <c r="C59" s="75"/>
-      <c r="D59" s="73"/>
-      <c r="E59" s="74"/>
-      <c r="F59" s="75"/>
-      <c r="G59" s="73"/>
-      <c r="H59" s="74"/>
-      <c r="I59" s="75"/>
+      <c r="A59" s="20"/>
+      <c r="B59" s="21"/>
+      <c r="C59" s="22"/>
+      <c r="D59" s="20"/>
+      <c r="E59" s="21"/>
+      <c r="F59" s="22"/>
+      <c r="G59" s="20"/>
+      <c r="H59" s="21"/>
+      <c r="I59" s="22"/>
       <c r="J59" s="1"/>
       <c r="K59" s="1"/>
       <c r="L59" s="1"/>
@@ -2773,15 +2800,15 @@
       <c r="Z59" s="1"/>
     </row>
     <row r="60" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A60" s="73"/>
-      <c r="B60" s="74"/>
-      <c r="C60" s="75"/>
-      <c r="D60" s="73"/>
-      <c r="E60" s="74"/>
-      <c r="F60" s="75"/>
-      <c r="G60" s="73"/>
-      <c r="H60" s="74"/>
-      <c r="I60" s="75"/>
+      <c r="A60" s="20"/>
+      <c r="B60" s="21"/>
+      <c r="C60" s="22"/>
+      <c r="D60" s="20"/>
+      <c r="E60" s="21"/>
+      <c r="F60" s="22"/>
+      <c r="G60" s="20"/>
+      <c r="H60" s="21"/>
+      <c r="I60" s="22"/>
       <c r="J60" s="1"/>
       <c r="K60" s="1"/>
       <c r="L60" s="1"/>
@@ -2801,15 +2828,15 @@
       <c r="Z60" s="1"/>
     </row>
     <row r="61" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A61" s="73"/>
-      <c r="B61" s="74"/>
-      <c r="C61" s="75"/>
-      <c r="D61" s="73"/>
-      <c r="E61" s="74"/>
-      <c r="F61" s="75"/>
-      <c r="G61" s="73"/>
-      <c r="H61" s="74"/>
-      <c r="I61" s="75"/>
+      <c r="A61" s="20"/>
+      <c r="B61" s="21"/>
+      <c r="C61" s="22"/>
+      <c r="D61" s="20"/>
+      <c r="E61" s="21"/>
+      <c r="F61" s="22"/>
+      <c r="G61" s="20"/>
+      <c r="H61" s="21"/>
+      <c r="I61" s="22"/>
       <c r="J61" s="1"/>
       <c r="K61" s="1"/>
       <c r="L61" s="1"/>
@@ -2829,15 +2856,15 @@
       <c r="Z61" s="1"/>
     </row>
     <row r="62" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A62" s="73"/>
-      <c r="B62" s="74"/>
-      <c r="C62" s="75"/>
-      <c r="D62" s="73"/>
-      <c r="E62" s="74"/>
-      <c r="F62" s="75"/>
-      <c r="G62" s="73"/>
-      <c r="H62" s="74"/>
-      <c r="I62" s="75"/>
+      <c r="A62" s="20"/>
+      <c r="B62" s="21"/>
+      <c r="C62" s="22"/>
+      <c r="D62" s="20"/>
+      <c r="E62" s="21"/>
+      <c r="F62" s="22"/>
+      <c r="G62" s="20"/>
+      <c r="H62" s="21"/>
+      <c r="I62" s="22"/>
       <c r="J62" s="1"/>
       <c r="K62" s="1"/>
       <c r="L62" s="1"/>
@@ -2857,15 +2884,15 @@
       <c r="Z62" s="1"/>
     </row>
     <row r="63" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A63" s="73"/>
-      <c r="B63" s="74"/>
-      <c r="C63" s="75"/>
-      <c r="D63" s="73"/>
-      <c r="E63" s="74"/>
-      <c r="F63" s="75"/>
-      <c r="G63" s="73"/>
-      <c r="H63" s="74"/>
-      <c r="I63" s="75"/>
+      <c r="A63" s="20"/>
+      <c r="B63" s="21"/>
+      <c r="C63" s="22"/>
+      <c r="D63" s="20"/>
+      <c r="E63" s="21"/>
+      <c r="F63" s="22"/>
+      <c r="G63" s="20"/>
+      <c r="H63" s="21"/>
+      <c r="I63" s="22"/>
       <c r="J63" s="1"/>
       <c r="K63" s="1"/>
       <c r="L63" s="1"/>
@@ -2885,15 +2912,15 @@
       <c r="Z63" s="1"/>
     </row>
     <row r="64" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A64" s="73"/>
-      <c r="B64" s="74"/>
-      <c r="C64" s="75"/>
-      <c r="D64" s="73"/>
-      <c r="E64" s="74"/>
-      <c r="F64" s="75"/>
-      <c r="G64" s="73"/>
-      <c r="H64" s="74"/>
-      <c r="I64" s="75"/>
+      <c r="A64" s="20"/>
+      <c r="B64" s="21"/>
+      <c r="C64" s="22"/>
+      <c r="D64" s="20"/>
+      <c r="E64" s="21"/>
+      <c r="F64" s="22"/>
+      <c r="G64" s="20"/>
+      <c r="H64" s="21"/>
+      <c r="I64" s="22"/>
       <c r="J64" s="1"/>
       <c r="K64" s="1"/>
       <c r="L64" s="1"/>
@@ -2913,15 +2940,15 @@
       <c r="Z64" s="1"/>
     </row>
     <row r="65" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A65" s="73"/>
-      <c r="B65" s="74"/>
-      <c r="C65" s="75"/>
-      <c r="D65" s="73"/>
-      <c r="E65" s="74"/>
-      <c r="F65" s="75"/>
-      <c r="G65" s="73"/>
-      <c r="H65" s="74"/>
-      <c r="I65" s="75"/>
+      <c r="A65" s="20"/>
+      <c r="B65" s="21"/>
+      <c r="C65" s="22"/>
+      <c r="D65" s="20"/>
+      <c r="E65" s="21"/>
+      <c r="F65" s="22"/>
+      <c r="G65" s="20"/>
+      <c r="H65" s="21"/>
+      <c r="I65" s="22"/>
       <c r="J65" s="1"/>
       <c r="K65" s="1"/>
       <c r="L65" s="1"/>
@@ -2941,15 +2968,15 @@
       <c r="Z65" s="1"/>
     </row>
     <row r="66" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A66" s="73"/>
-      <c r="B66" s="74"/>
-      <c r="C66" s="75"/>
-      <c r="D66" s="73"/>
-      <c r="E66" s="74"/>
-      <c r="F66" s="75"/>
-      <c r="G66" s="73"/>
-      <c r="H66" s="74"/>
-      <c r="I66" s="75"/>
+      <c r="A66" s="20"/>
+      <c r="B66" s="21"/>
+      <c r="C66" s="22"/>
+      <c r="D66" s="20"/>
+      <c r="E66" s="21"/>
+      <c r="F66" s="22"/>
+      <c r="G66" s="20"/>
+      <c r="H66" s="21"/>
+      <c r="I66" s="22"/>
       <c r="J66" s="1"/>
       <c r="K66" s="1"/>
       <c r="L66" s="1"/>
@@ -2969,15 +2996,15 @@
       <c r="Z66" s="1"/>
     </row>
     <row r="67" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A67" s="73"/>
-      <c r="B67" s="74"/>
-      <c r="C67" s="75"/>
-      <c r="D67" s="76"/>
-      <c r="E67" s="77"/>
-      <c r="F67" s="78"/>
-      <c r="G67" s="76"/>
-      <c r="H67" s="77"/>
-      <c r="I67" s="78"/>
+      <c r="A67" s="20"/>
+      <c r="B67" s="21"/>
+      <c r="C67" s="22"/>
+      <c r="D67" s="23"/>
+      <c r="E67" s="24"/>
+      <c r="F67" s="25"/>
+      <c r="G67" s="23"/>
+      <c r="H67" s="24"/>
+      <c r="I67" s="25"/>
       <c r="J67" s="1"/>
       <c r="K67" s="1"/>
       <c r="L67" s="1"/>
@@ -2997,21 +3024,21 @@
       <c r="Z67" s="1"/>
     </row>
     <row r="68" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A68" s="38" t="s">
+      <c r="A68" s="40" t="s">
         <v>33</v>
       </c>
-      <c r="B68" s="29"/>
-      <c r="C68" s="30"/>
-      <c r="D68" s="38" t="s">
+      <c r="B68" s="33"/>
+      <c r="C68" s="34"/>
+      <c r="D68" s="40" t="s">
         <v>34</v>
       </c>
-      <c r="E68" s="29"/>
-      <c r="F68" s="30"/>
-      <c r="G68" s="39" t="s">
+      <c r="E68" s="33"/>
+      <c r="F68" s="34"/>
+      <c r="G68" s="49" t="s">
         <v>35</v>
       </c>
-      <c r="H68" s="29"/>
-      <c r="I68" s="30"/>
+      <c r="H68" s="33"/>
+      <c r="I68" s="34"/>
       <c r="J68" s="1"/>
       <c r="K68" s="1"/>
       <c r="L68" s="1"/>
@@ -3031,15 +3058,15 @@
       <c r="Z68" s="1"/>
     </row>
     <row r="69" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A69" s="70"/>
-      <c r="B69" s="71"/>
-      <c r="C69" s="72"/>
-      <c r="D69" s="70"/>
-      <c r="E69" s="71"/>
-      <c r="F69" s="72"/>
-      <c r="G69" s="79"/>
-      <c r="H69" s="71"/>
-      <c r="I69" s="72"/>
+      <c r="A69" s="17"/>
+      <c r="B69" s="18"/>
+      <c r="C69" s="19"/>
+      <c r="D69" s="17"/>
+      <c r="E69" s="18"/>
+      <c r="F69" s="19"/>
+      <c r="G69" s="26"/>
+      <c r="H69" s="18"/>
+      <c r="I69" s="19"/>
       <c r="J69" s="1"/>
       <c r="K69" s="1"/>
       <c r="L69" s="1"/>
@@ -3059,15 +3086,15 @@
       <c r="Z69" s="1"/>
     </row>
     <row r="70" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A70" s="73"/>
-      <c r="B70" s="74"/>
-      <c r="C70" s="75"/>
-      <c r="D70" s="73"/>
-      <c r="E70" s="74"/>
-      <c r="F70" s="75"/>
-      <c r="G70" s="73"/>
-      <c r="H70" s="74"/>
-      <c r="I70" s="75"/>
+      <c r="A70" s="20"/>
+      <c r="B70" s="21"/>
+      <c r="C70" s="22"/>
+      <c r="D70" s="20"/>
+      <c r="E70" s="21"/>
+      <c r="F70" s="22"/>
+      <c r="G70" s="20"/>
+      <c r="H70" s="21"/>
+      <c r="I70" s="22"/>
       <c r="J70" s="1"/>
       <c r="K70" s="1"/>
       <c r="L70" s="1"/>
@@ -3087,15 +3114,15 @@
       <c r="Z70" s="1"/>
     </row>
     <row r="71" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A71" s="73"/>
-      <c r="B71" s="74"/>
-      <c r="C71" s="75"/>
-      <c r="D71" s="73"/>
-      <c r="E71" s="74"/>
-      <c r="F71" s="75"/>
-      <c r="G71" s="73"/>
-      <c r="H71" s="74"/>
-      <c r="I71" s="75"/>
+      <c r="A71" s="20"/>
+      <c r="B71" s="21"/>
+      <c r="C71" s="22"/>
+      <c r="D71" s="20"/>
+      <c r="E71" s="21"/>
+      <c r="F71" s="22"/>
+      <c r="G71" s="20"/>
+      <c r="H71" s="21"/>
+      <c r="I71" s="22"/>
       <c r="J71" s="1"/>
       <c r="K71" s="1"/>
       <c r="L71" s="1"/>
@@ -3115,15 +3142,15 @@
       <c r="Z71" s="1"/>
     </row>
     <row r="72" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A72" s="73"/>
-      <c r="B72" s="74"/>
-      <c r="C72" s="75"/>
-      <c r="D72" s="73"/>
-      <c r="E72" s="74"/>
-      <c r="F72" s="75"/>
-      <c r="G72" s="73"/>
-      <c r="H72" s="74"/>
-      <c r="I72" s="75"/>
+      <c r="A72" s="20"/>
+      <c r="B72" s="21"/>
+      <c r="C72" s="22"/>
+      <c r="D72" s="20"/>
+      <c r="E72" s="21"/>
+      <c r="F72" s="22"/>
+      <c r="G72" s="20"/>
+      <c r="H72" s="21"/>
+      <c r="I72" s="22"/>
       <c r="J72" s="1"/>
       <c r="K72" s="1"/>
       <c r="L72" s="1"/>
@@ -3143,15 +3170,15 @@
       <c r="Z72" s="1"/>
     </row>
     <row r="73" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A73" s="73"/>
-      <c r="B73" s="74"/>
-      <c r="C73" s="75"/>
-      <c r="D73" s="73"/>
-      <c r="E73" s="74"/>
-      <c r="F73" s="75"/>
-      <c r="G73" s="73"/>
-      <c r="H73" s="74"/>
-      <c r="I73" s="75"/>
+      <c r="A73" s="20"/>
+      <c r="B73" s="21"/>
+      <c r="C73" s="22"/>
+      <c r="D73" s="20"/>
+      <c r="E73" s="21"/>
+      <c r="F73" s="22"/>
+      <c r="G73" s="20"/>
+      <c r="H73" s="21"/>
+      <c r="I73" s="22"/>
       <c r="J73" s="1"/>
       <c r="K73" s="1"/>
       <c r="L73" s="1"/>
@@ -3171,15 +3198,15 @@
       <c r="Z73" s="1"/>
     </row>
     <row r="74" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A74" s="73"/>
-      <c r="B74" s="74"/>
-      <c r="C74" s="75"/>
-      <c r="D74" s="73"/>
-      <c r="E74" s="74"/>
-      <c r="F74" s="75"/>
-      <c r="G74" s="73"/>
-      <c r="H74" s="74"/>
-      <c r="I74" s="75"/>
+      <c r="A74" s="20"/>
+      <c r="B74" s="21"/>
+      <c r="C74" s="22"/>
+      <c r="D74" s="20"/>
+      <c r="E74" s="21"/>
+      <c r="F74" s="22"/>
+      <c r="G74" s="20"/>
+      <c r="H74" s="21"/>
+      <c r="I74" s="22"/>
       <c r="J74" s="1"/>
       <c r="K74" s="1"/>
       <c r="L74" s="1"/>
@@ -3199,15 +3226,15 @@
       <c r="Z74" s="1"/>
     </row>
     <row r="75" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A75" s="73"/>
-      <c r="B75" s="74"/>
-      <c r="C75" s="75"/>
-      <c r="D75" s="73"/>
-      <c r="E75" s="74"/>
-      <c r="F75" s="75"/>
-      <c r="G75" s="73"/>
-      <c r="H75" s="74"/>
-      <c r="I75" s="75"/>
+      <c r="A75" s="20"/>
+      <c r="B75" s="21"/>
+      <c r="C75" s="22"/>
+      <c r="D75" s="20"/>
+      <c r="E75" s="21"/>
+      <c r="F75" s="22"/>
+      <c r="G75" s="20"/>
+      <c r="H75" s="21"/>
+      <c r="I75" s="22"/>
       <c r="J75" s="1"/>
       <c r="K75" s="1"/>
       <c r="L75" s="1"/>
@@ -3227,15 +3254,15 @@
       <c r="Z75" s="1"/>
     </row>
     <row r="76" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A76" s="73"/>
-      <c r="B76" s="74"/>
-      <c r="C76" s="75"/>
-      <c r="D76" s="73"/>
-      <c r="E76" s="74"/>
-      <c r="F76" s="75"/>
-      <c r="G76" s="73"/>
-      <c r="H76" s="74"/>
-      <c r="I76" s="75"/>
+      <c r="A76" s="20"/>
+      <c r="B76" s="21"/>
+      <c r="C76" s="22"/>
+      <c r="D76" s="20"/>
+      <c r="E76" s="21"/>
+      <c r="F76" s="22"/>
+      <c r="G76" s="20"/>
+      <c r="H76" s="21"/>
+      <c r="I76" s="22"/>
       <c r="J76" s="1"/>
       <c r="K76" s="1"/>
       <c r="L76" s="1"/>
@@ -3255,15 +3282,15 @@
       <c r="Z76" s="1"/>
     </row>
     <row r="77" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A77" s="73"/>
-      <c r="B77" s="74"/>
-      <c r="C77" s="75"/>
-      <c r="D77" s="73"/>
-      <c r="E77" s="74"/>
-      <c r="F77" s="75"/>
-      <c r="G77" s="73"/>
-      <c r="H77" s="74"/>
-      <c r="I77" s="75"/>
+      <c r="A77" s="20"/>
+      <c r="B77" s="21"/>
+      <c r="C77" s="22"/>
+      <c r="D77" s="20"/>
+      <c r="E77" s="21"/>
+      <c r="F77" s="22"/>
+      <c r="G77" s="20"/>
+      <c r="H77" s="21"/>
+      <c r="I77" s="22"/>
       <c r="J77" s="1"/>
       <c r="K77" s="1"/>
       <c r="L77" s="1"/>
@@ -3283,15 +3310,15 @@
       <c r="Z77" s="1"/>
     </row>
     <row r="78" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A78" s="73"/>
-      <c r="B78" s="74"/>
-      <c r="C78" s="75"/>
-      <c r="D78" s="76"/>
-      <c r="E78" s="77"/>
-      <c r="F78" s="78"/>
-      <c r="G78" s="76"/>
-      <c r="H78" s="77"/>
-      <c r="I78" s="78"/>
+      <c r="A78" s="20"/>
+      <c r="B78" s="21"/>
+      <c r="C78" s="22"/>
+      <c r="D78" s="23"/>
+      <c r="E78" s="24"/>
+      <c r="F78" s="25"/>
+      <c r="G78" s="23"/>
+      <c r="H78" s="24"/>
+      <c r="I78" s="25"/>
       <c r="J78" s="1"/>
       <c r="K78" s="1"/>
       <c r="L78" s="1"/>
@@ -3311,15 +3338,15 @@
       <c r="Z78" s="1"/>
     </row>
     <row r="79" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A79" s="73"/>
-      <c r="B79" s="74"/>
-      <c r="C79" s="75"/>
-      <c r="D79" s="70"/>
-      <c r="E79" s="71"/>
-      <c r="F79" s="72"/>
-      <c r="G79" s="70"/>
-      <c r="H79" s="71"/>
-      <c r="I79" s="72"/>
+      <c r="A79" s="20"/>
+      <c r="B79" s="21"/>
+      <c r="C79" s="22"/>
+      <c r="D79" s="17"/>
+      <c r="E79" s="18"/>
+      <c r="F79" s="19"/>
+      <c r="G79" s="17"/>
+      <c r="H79" s="18"/>
+      <c r="I79" s="19"/>
       <c r="J79" s="1"/>
       <c r="K79" s="1"/>
       <c r="L79" s="1"/>
@@ -3339,15 +3366,15 @@
       <c r="Z79" s="1"/>
     </row>
     <row r="80" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A80" s="73"/>
-      <c r="B80" s="74"/>
-      <c r="C80" s="75"/>
-      <c r="D80" s="73"/>
-      <c r="E80" s="74"/>
-      <c r="F80" s="75"/>
-      <c r="G80" s="73"/>
-      <c r="H80" s="74"/>
-      <c r="I80" s="75"/>
+      <c r="A80" s="20"/>
+      <c r="B80" s="21"/>
+      <c r="C80" s="22"/>
+      <c r="D80" s="20"/>
+      <c r="E80" s="21"/>
+      <c r="F80" s="22"/>
+      <c r="G80" s="20"/>
+      <c r="H80" s="21"/>
+      <c r="I80" s="22"/>
       <c r="J80" s="1"/>
       <c r="K80" s="1"/>
       <c r="L80" s="1"/>
@@ -3367,15 +3394,15 @@
       <c r="Z80" s="1"/>
     </row>
     <row r="81" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A81" s="73"/>
-      <c r="B81" s="74"/>
-      <c r="C81" s="75"/>
-      <c r="D81" s="73"/>
-      <c r="E81" s="74"/>
-      <c r="F81" s="75"/>
-      <c r="G81" s="73"/>
-      <c r="H81" s="74"/>
-      <c r="I81" s="75"/>
+      <c r="A81" s="20"/>
+      <c r="B81" s="21"/>
+      <c r="C81" s="22"/>
+      <c r="D81" s="20"/>
+      <c r="E81" s="21"/>
+      <c r="F81" s="22"/>
+      <c r="G81" s="20"/>
+      <c r="H81" s="21"/>
+      <c r="I81" s="22"/>
       <c r="J81" s="1"/>
       <c r="K81" s="1"/>
       <c r="L81" s="1"/>
@@ -3395,15 +3422,15 @@
       <c r="Z81" s="1"/>
     </row>
     <row r="82" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A82" s="73"/>
-      <c r="B82" s="74"/>
-      <c r="C82" s="75"/>
-      <c r="D82" s="73"/>
-      <c r="E82" s="74"/>
-      <c r="F82" s="75"/>
-      <c r="G82" s="73"/>
-      <c r="H82" s="74"/>
-      <c r="I82" s="75"/>
+      <c r="A82" s="20"/>
+      <c r="B82" s="21"/>
+      <c r="C82" s="22"/>
+      <c r="D82" s="20"/>
+      <c r="E82" s="21"/>
+      <c r="F82" s="22"/>
+      <c r="G82" s="20"/>
+      <c r="H82" s="21"/>
+      <c r="I82" s="22"/>
       <c r="J82" s="1"/>
       <c r="K82" s="1"/>
       <c r="L82" s="1"/>
@@ -3423,15 +3450,15 @@
       <c r="Z82" s="1"/>
     </row>
     <row r="83" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A83" s="73"/>
-      <c r="B83" s="74"/>
-      <c r="C83" s="75"/>
-      <c r="D83" s="73"/>
-      <c r="E83" s="74"/>
-      <c r="F83" s="75"/>
-      <c r="G83" s="73"/>
-      <c r="H83" s="74"/>
-      <c r="I83" s="75"/>
+      <c r="A83" s="20"/>
+      <c r="B83" s="21"/>
+      <c r="C83" s="22"/>
+      <c r="D83" s="20"/>
+      <c r="E83" s="21"/>
+      <c r="F83" s="22"/>
+      <c r="G83" s="20"/>
+      <c r="H83" s="21"/>
+      <c r="I83" s="22"/>
       <c r="J83" s="1"/>
       <c r="K83" s="1"/>
       <c r="L83" s="1"/>
@@ -3451,15 +3478,15 @@
       <c r="Z83" s="1"/>
     </row>
     <row r="84" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A84" s="73"/>
-      <c r="B84" s="74"/>
-      <c r="C84" s="75"/>
-      <c r="D84" s="73"/>
-      <c r="E84" s="74"/>
-      <c r="F84" s="75"/>
-      <c r="G84" s="73"/>
-      <c r="H84" s="74"/>
-      <c r="I84" s="75"/>
+      <c r="A84" s="20"/>
+      <c r="B84" s="21"/>
+      <c r="C84" s="22"/>
+      <c r="D84" s="20"/>
+      <c r="E84" s="21"/>
+      <c r="F84" s="22"/>
+      <c r="G84" s="20"/>
+      <c r="H84" s="21"/>
+      <c r="I84" s="22"/>
       <c r="J84" s="1"/>
       <c r="K84" s="1"/>
       <c r="L84" s="1"/>
@@ -3479,15 +3506,15 @@
       <c r="Z84" s="1"/>
     </row>
     <row r="85" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A85" s="73"/>
-      <c r="B85" s="74"/>
-      <c r="C85" s="75"/>
-      <c r="D85" s="73"/>
-      <c r="E85" s="74"/>
-      <c r="F85" s="75"/>
-      <c r="G85" s="73"/>
-      <c r="H85" s="74"/>
-      <c r="I85" s="75"/>
+      <c r="A85" s="20"/>
+      <c r="B85" s="21"/>
+      <c r="C85" s="22"/>
+      <c r="D85" s="20"/>
+      <c r="E85" s="21"/>
+      <c r="F85" s="22"/>
+      <c r="G85" s="20"/>
+      <c r="H85" s="21"/>
+      <c r="I85" s="22"/>
       <c r="J85" s="1"/>
       <c r="K85" s="1"/>
       <c r="L85" s="1"/>
@@ -3507,15 +3534,15 @@
       <c r="Z85" s="1"/>
     </row>
     <row r="86" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A86" s="73"/>
-      <c r="B86" s="74"/>
-      <c r="C86" s="75"/>
-      <c r="D86" s="73"/>
-      <c r="E86" s="74"/>
-      <c r="F86" s="75"/>
-      <c r="G86" s="73"/>
-      <c r="H86" s="74"/>
-      <c r="I86" s="75"/>
+      <c r="A86" s="20"/>
+      <c r="B86" s="21"/>
+      <c r="C86" s="22"/>
+      <c r="D86" s="20"/>
+      <c r="E86" s="21"/>
+      <c r="F86" s="22"/>
+      <c r="G86" s="20"/>
+      <c r="H86" s="21"/>
+      <c r="I86" s="22"/>
       <c r="J86" s="1"/>
       <c r="K86" s="1"/>
       <c r="L86" s="1"/>
@@ -3535,15 +3562,15 @@
       <c r="Z86" s="1"/>
     </row>
     <row r="87" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A87" s="73"/>
-      <c r="B87" s="74"/>
-      <c r="C87" s="75"/>
-      <c r="D87" s="73"/>
-      <c r="E87" s="74"/>
-      <c r="F87" s="75"/>
-      <c r="G87" s="73"/>
-      <c r="H87" s="74"/>
-      <c r="I87" s="75"/>
+      <c r="A87" s="20"/>
+      <c r="B87" s="21"/>
+      <c r="C87" s="22"/>
+      <c r="D87" s="20"/>
+      <c r="E87" s="21"/>
+      <c r="F87" s="22"/>
+      <c r="G87" s="20"/>
+      <c r="H87" s="21"/>
+      <c r="I87" s="22"/>
       <c r="J87" s="1"/>
       <c r="K87" s="1"/>
       <c r="L87" s="1"/>
@@ -3563,15 +3590,15 @@
       <c r="Z87" s="1"/>
     </row>
     <row r="88" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A88" s="76"/>
-      <c r="B88" s="77"/>
-      <c r="C88" s="78"/>
-      <c r="D88" s="76"/>
-      <c r="E88" s="77"/>
-      <c r="F88" s="78"/>
-      <c r="G88" s="76"/>
-      <c r="H88" s="77"/>
-      <c r="I88" s="78"/>
+      <c r="A88" s="23"/>
+      <c r="B88" s="24"/>
+      <c r="C88" s="25"/>
+      <c r="D88" s="23"/>
+      <c r="E88" s="24"/>
+      <c r="F88" s="25"/>
+      <c r="G88" s="23"/>
+      <c r="H88" s="24"/>
+      <c r="I88" s="25"/>
       <c r="J88" s="1"/>
       <c r="K88" s="1"/>
       <c r="L88" s="1"/>
@@ -3591,21 +3618,21 @@
       <c r="Z88" s="1"/>
     </row>
     <row r="89" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A89" s="38" t="s">
+      <c r="A89" s="40" t="s">
         <v>36</v>
       </c>
-      <c r="B89" s="29"/>
-      <c r="C89" s="30"/>
-      <c r="D89" s="38" t="s">
+      <c r="B89" s="33"/>
+      <c r="C89" s="34"/>
+      <c r="D89" s="40" t="s">
         <v>37</v>
       </c>
-      <c r="E89" s="29"/>
-      <c r="F89" s="30"/>
-      <c r="G89" s="38" t="s">
+      <c r="E89" s="33"/>
+      <c r="F89" s="34"/>
+      <c r="G89" s="40" t="s">
         <v>38</v>
       </c>
-      <c r="H89" s="29"/>
-      <c r="I89" s="30"/>
+      <c r="H89" s="33"/>
+      <c r="I89" s="34"/>
       <c r="J89" s="1"/>
       <c r="K89" s="1"/>
       <c r="L89" s="1"/>
@@ -3626,14 +3653,14 @@
     </row>
     <row r="90" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A90" s="41"/>
-      <c r="B90" s="42"/>
-      <c r="C90" s="42"/>
-      <c r="D90" s="42"/>
-      <c r="E90" s="42"/>
-      <c r="F90" s="42"/>
-      <c r="G90" s="42"/>
-      <c r="H90" s="42"/>
-      <c r="I90" s="42"/>
+      <c r="B90" s="38"/>
+      <c r="C90" s="38"/>
+      <c r="D90" s="38"/>
+      <c r="E90" s="38"/>
+      <c r="F90" s="38"/>
+      <c r="G90" s="38"/>
+      <c r="H90" s="38"/>
+      <c r="I90" s="38"/>
       <c r="J90" s="1"/>
       <c r="K90" s="1"/>
       <c r="L90" s="1"/>
@@ -3653,19 +3680,19 @@
       <c r="Z90" s="1"/>
     </row>
     <row r="91" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A91" s="43" t="s">
+      <c r="A91" s="42" t="s">
         <v>39</v>
       </c>
-      <c r="B91" s="24"/>
-      <c r="C91" s="25"/>
-      <c r="D91" s="44"/>
-      <c r="E91" s="42"/>
-      <c r="F91" s="45" t="s">
+      <c r="B91" s="43"/>
+      <c r="C91" s="44"/>
+      <c r="D91" s="45"/>
+      <c r="E91" s="38"/>
+      <c r="F91" s="46" t="s">
         <v>40</v>
       </c>
-      <c r="G91" s="42"/>
-      <c r="H91" s="42"/>
-      <c r="I91" s="26"/>
+      <c r="G91" s="38"/>
+      <c r="H91" s="38"/>
+      <c r="I91" s="47"/>
       <c r="J91" s="1"/>
       <c r="K91" s="1"/>
       <c r="L91" s="1"/>
@@ -3694,16 +3721,16 @@
       <c r="C92" s="3" t="s">
         <v>43</v>
       </c>
-      <c r="D92" s="42"/>
-      <c r="E92" s="42"/>
+      <c r="D92" s="38"/>
+      <c r="E92" s="38"/>
       <c r="F92" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="G92" s="28" t="s">
+      <c r="G92" s="35" t="s">
         <v>44</v>
       </c>
-      <c r="H92" s="29"/>
-      <c r="I92" s="30"/>
+      <c r="H92" s="33"/>
+      <c r="I92" s="34"/>
       <c r="J92" s="1"/>
       <c r="K92" s="1"/>
       <c r="L92" s="1"/>
@@ -3728,12 +3755,12 @@
       </c>
       <c r="B93" s="8"/>
       <c r="C93" s="8"/>
-      <c r="D93" s="42"/>
-      <c r="E93" s="42"/>
+      <c r="D93" s="38"/>
+      <c r="E93" s="38"/>
       <c r="F93" s="4"/>
-      <c r="G93" s="46"/>
-      <c r="H93" s="29"/>
-      <c r="I93" s="30"/>
+      <c r="G93" s="48"/>
+      <c r="H93" s="33"/>
+      <c r="I93" s="34"/>
       <c r="J93" s="1"/>
       <c r="K93" s="1"/>
       <c r="L93" s="1"/>
@@ -3758,12 +3785,12 @@
       </c>
       <c r="B94" s="8"/>
       <c r="C94" s="8"/>
-      <c r="D94" s="42"/>
-      <c r="E94" s="42"/>
+      <c r="D94" s="38"/>
+      <c r="E94" s="38"/>
       <c r="F94" s="4"/>
-      <c r="G94" s="46"/>
-      <c r="H94" s="29"/>
-      <c r="I94" s="30"/>
+      <c r="G94" s="48"/>
+      <c r="H94" s="33"/>
+      <c r="I94" s="34"/>
       <c r="J94" s="1"/>
       <c r="K94" s="1"/>
       <c r="L94" s="1"/>
@@ -3788,12 +3815,12 @@
       </c>
       <c r="B95" s="8"/>
       <c r="C95" s="8"/>
-      <c r="D95" s="42"/>
-      <c r="E95" s="42"/>
+      <c r="D95" s="38"/>
+      <c r="E95" s="38"/>
       <c r="F95" s="4"/>
-      <c r="G95" s="46"/>
-      <c r="H95" s="29"/>
-      <c r="I95" s="30"/>
+      <c r="G95" s="48"/>
+      <c r="H95" s="33"/>
+      <c r="I95" s="34"/>
       <c r="J95" s="1"/>
       <c r="K95" s="1"/>
       <c r="L95" s="1"/>
@@ -3818,12 +3845,12 @@
       </c>
       <c r="B96" s="8"/>
       <c r="C96" s="8"/>
-      <c r="D96" s="42"/>
-      <c r="E96" s="42"/>
+      <c r="D96" s="38"/>
+      <c r="E96" s="38"/>
       <c r="F96" s="4"/>
-      <c r="G96" s="46"/>
-      <c r="H96" s="29"/>
-      <c r="I96" s="30"/>
+      <c r="G96" s="48"/>
+      <c r="H96" s="33"/>
+      <c r="I96" s="34"/>
       <c r="J96" s="1"/>
       <c r="K96" s="1"/>
       <c r="L96" s="1"/>
@@ -3848,12 +3875,12 @@
       </c>
       <c r="B97" s="8"/>
       <c r="C97" s="8"/>
-      <c r="D97" s="42"/>
-      <c r="E97" s="42"/>
+      <c r="D97" s="38"/>
+      <c r="E97" s="38"/>
       <c r="F97" s="4"/>
-      <c r="G97" s="46"/>
-      <c r="H97" s="29"/>
-      <c r="I97" s="30"/>
+      <c r="G97" s="48"/>
+      <c r="H97" s="33"/>
+      <c r="I97" s="34"/>
       <c r="J97" s="1"/>
       <c r="K97" s="1"/>
       <c r="L97" s="1"/>
@@ -3878,12 +3905,12 @@
       </c>
       <c r="B98" s="8"/>
       <c r="C98" s="8"/>
-      <c r="D98" s="42"/>
-      <c r="E98" s="42"/>
+      <c r="D98" s="38"/>
+      <c r="E98" s="38"/>
       <c r="F98" s="4"/>
-      <c r="G98" s="46"/>
-      <c r="H98" s="29"/>
-      <c r="I98" s="30"/>
+      <c r="G98" s="48"/>
+      <c r="H98" s="33"/>
+      <c r="I98" s="34"/>
       <c r="J98" s="1"/>
       <c r="K98" s="1"/>
       <c r="L98" s="1"/>
@@ -3908,12 +3935,12 @@
       </c>
       <c r="B99" s="8"/>
       <c r="C99" s="8"/>
-      <c r="D99" s="42"/>
-      <c r="E99" s="42"/>
+      <c r="D99" s="38"/>
+      <c r="E99" s="38"/>
       <c r="F99" s="4"/>
-      <c r="G99" s="46"/>
-      <c r="H99" s="29"/>
-      <c r="I99" s="30"/>
+      <c r="G99" s="48"/>
+      <c r="H99" s="33"/>
+      <c r="I99" s="34"/>
       <c r="J99" s="1"/>
       <c r="K99" s="1"/>
       <c r="L99" s="1"/>
@@ -3936,14 +3963,14 @@
       <c r="A100" s="3" t="s">
         <v>52</v>
       </c>
-      <c r="B100" s="47"/>
-      <c r="C100" s="30"/>
-      <c r="D100" s="48"/>
-      <c r="E100" s="48"/>
-      <c r="F100" s="42"/>
-      <c r="G100" s="42"/>
-      <c r="H100" s="42"/>
-      <c r="I100" s="42"/>
+      <c r="B100" s="36"/>
+      <c r="C100" s="34"/>
+      <c r="D100" s="37"/>
+      <c r="E100" s="37"/>
+      <c r="F100" s="38"/>
+      <c r="G100" s="38"/>
+      <c r="H100" s="38"/>
+      <c r="I100" s="38"/>
       <c r="J100" s="1"/>
       <c r="K100" s="1"/>
       <c r="L100" s="1"/>
@@ -3963,15 +3990,15 @@
       <c r="Z100" s="1"/>
     </row>
     <row r="101" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A101" s="48"/>
-      <c r="B101" s="42"/>
-      <c r="C101" s="42"/>
-      <c r="D101" s="42"/>
-      <c r="E101" s="42"/>
-      <c r="F101" s="42"/>
-      <c r="G101" s="42"/>
-      <c r="H101" s="42"/>
-      <c r="I101" s="42"/>
+      <c r="A101" s="37"/>
+      <c r="B101" s="38"/>
+      <c r="C101" s="38"/>
+      <c r="D101" s="38"/>
+      <c r="E101" s="38"/>
+      <c r="F101" s="38"/>
+      <c r="G101" s="38"/>
+      <c r="H101" s="38"/>
+      <c r="I101" s="38"/>
       <c r="J101" s="1"/>
       <c r="K101" s="1"/>
       <c r="L101" s="1"/>
@@ -3991,17 +4018,17 @@
       <c r="Z101" s="1"/>
     </row>
     <row r="102" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A102" s="49" t="s">
+      <c r="A102" s="39" t="s">
         <v>53</v>
       </c>
-      <c r="B102" s="21"/>
-      <c r="C102" s="21"/>
-      <c r="D102" s="21"/>
-      <c r="E102" s="21"/>
-      <c r="F102" s="21"/>
-      <c r="G102" s="21"/>
-      <c r="H102" s="21"/>
-      <c r="I102" s="22"/>
+      <c r="B102" s="29"/>
+      <c r="C102" s="29"/>
+      <c r="D102" s="29"/>
+      <c r="E102" s="29"/>
+      <c r="F102" s="29"/>
+      <c r="G102" s="29"/>
+      <c r="H102" s="29"/>
+      <c r="I102" s="30"/>
       <c r="J102" s="1"/>
       <c r="K102" s="1"/>
       <c r="L102" s="1"/>
@@ -4024,14 +4051,14 @@
       <c r="A103" s="3" t="s">
         <v>54</v>
       </c>
-      <c r="B103" s="28" t="s">
+      <c r="B103" s="35" t="s">
         <v>55</v>
       </c>
-      <c r="C103" s="29"/>
-      <c r="D103" s="29"/>
-      <c r="E103" s="29"/>
-      <c r="F103" s="29"/>
-      <c r="G103" s="29"/>
+      <c r="C103" s="33"/>
+      <c r="D103" s="33"/>
+      <c r="E103" s="33"/>
+      <c r="F103" s="33"/>
+      <c r="G103" s="33"/>
       <c r="H103" s="3" t="s">
         <v>56</v>
       </c>
@@ -4060,14 +4087,14 @@
       <c r="A104" s="9">
         <v>1</v>
       </c>
-      <c r="B104" s="50" t="s">
+      <c r="B104" s="32" t="s">
         <v>58</v>
       </c>
-      <c r="C104" s="29"/>
-      <c r="D104" s="29"/>
-      <c r="E104" s="29"/>
-      <c r="F104" s="29"/>
-      <c r="G104" s="30"/>
+      <c r="C104" s="33"/>
+      <c r="D104" s="33"/>
+      <c r="E104" s="33"/>
+      <c r="F104" s="33"/>
+      <c r="G104" s="34"/>
       <c r="H104" s="4"/>
       <c r="I104" s="4"/>
       <c r="J104" s="1"/>
@@ -4092,14 +4119,14 @@
       <c r="A105" s="9">
         <v>2</v>
       </c>
-      <c r="B105" s="50" t="s">
+      <c r="B105" s="32" t="s">
         <v>59</v>
       </c>
-      <c r="C105" s="29"/>
-      <c r="D105" s="29"/>
-      <c r="E105" s="29"/>
-      <c r="F105" s="29"/>
-      <c r="G105" s="30"/>
+      <c r="C105" s="33"/>
+      <c r="D105" s="33"/>
+      <c r="E105" s="33"/>
+      <c r="F105" s="33"/>
+      <c r="G105" s="34"/>
       <c r="H105" s="4"/>
       <c r="I105" s="4"/>
       <c r="J105" s="1"/>
@@ -4124,14 +4151,14 @@
       <c r="A106" s="9">
         <v>3</v>
       </c>
-      <c r="B106" s="50" t="s">
+      <c r="B106" s="32" t="s">
         <v>60</v>
       </c>
-      <c r="C106" s="29"/>
-      <c r="D106" s="29"/>
-      <c r="E106" s="29"/>
-      <c r="F106" s="29"/>
-      <c r="G106" s="30"/>
+      <c r="C106" s="33"/>
+      <c r="D106" s="33"/>
+      <c r="E106" s="33"/>
+      <c r="F106" s="33"/>
+      <c r="G106" s="34"/>
       <c r="H106" s="4"/>
       <c r="I106" s="4"/>
       <c r="J106" s="1"/>
@@ -4156,14 +4183,14 @@
       <c r="A107" s="9">
         <v>4</v>
       </c>
-      <c r="B107" s="50" t="s">
+      <c r="B107" s="32" t="s">
         <v>61</v>
       </c>
-      <c r="C107" s="29"/>
-      <c r="D107" s="29"/>
-      <c r="E107" s="29"/>
-      <c r="F107" s="29"/>
-      <c r="G107" s="30"/>
+      <c r="C107" s="33"/>
+      <c r="D107" s="33"/>
+      <c r="E107" s="33"/>
+      <c r="F107" s="33"/>
+      <c r="G107" s="34"/>
       <c r="H107" s="4"/>
       <c r="I107" s="4"/>
       <c r="J107" s="1"/>
@@ -4188,14 +4215,14 @@
       <c r="A108" s="9">
         <v>5</v>
       </c>
-      <c r="B108" s="50" t="s">
+      <c r="B108" s="32" t="s">
         <v>62</v>
       </c>
-      <c r="C108" s="29"/>
-      <c r="D108" s="29"/>
-      <c r="E108" s="29"/>
-      <c r="F108" s="29"/>
-      <c r="G108" s="30"/>
+      <c r="C108" s="33"/>
+      <c r="D108" s="33"/>
+      <c r="E108" s="33"/>
+      <c r="F108" s="33"/>
+      <c r="G108" s="34"/>
       <c r="H108" s="4"/>
       <c r="I108" s="4"/>
       <c r="J108" s="1"/>
@@ -4220,14 +4247,14 @@
       <c r="A109" s="9">
         <v>6</v>
       </c>
-      <c r="B109" s="50" t="s">
+      <c r="B109" s="32" t="s">
         <v>63</v>
       </c>
-      <c r="C109" s="29"/>
-      <c r="D109" s="29"/>
-      <c r="E109" s="29"/>
-      <c r="F109" s="29"/>
-      <c r="G109" s="30"/>
+      <c r="C109" s="33"/>
+      <c r="D109" s="33"/>
+      <c r="E109" s="33"/>
+      <c r="F109" s="33"/>
+      <c r="G109" s="34"/>
       <c r="H109" s="4"/>
       <c r="I109" s="4"/>
       <c r="J109" s="1"/>
@@ -4252,14 +4279,14 @@
       <c r="A110" s="9">
         <v>7</v>
       </c>
-      <c r="B110" s="50" t="s">
+      <c r="B110" s="32" t="s">
         <v>64</v>
       </c>
-      <c r="C110" s="29"/>
-      <c r="D110" s="29"/>
-      <c r="E110" s="29"/>
-      <c r="F110" s="29"/>
-      <c r="G110" s="30"/>
+      <c r="C110" s="33"/>
+      <c r="D110" s="33"/>
+      <c r="E110" s="33"/>
+      <c r="F110" s="33"/>
+      <c r="G110" s="34"/>
       <c r="H110" s="4"/>
       <c r="I110" s="4"/>
       <c r="J110" s="1"/>
@@ -4284,14 +4311,14 @@
       <c r="A111" s="9">
         <v>8</v>
       </c>
-      <c r="B111" s="50" t="s">
+      <c r="B111" s="32" t="s">
         <v>65</v>
       </c>
-      <c r="C111" s="29"/>
-      <c r="D111" s="29"/>
-      <c r="E111" s="29"/>
-      <c r="F111" s="29"/>
-      <c r="G111" s="30"/>
+      <c r="C111" s="33"/>
+      <c r="D111" s="33"/>
+      <c r="E111" s="33"/>
+      <c r="F111" s="33"/>
+      <c r="G111" s="34"/>
       <c r="H111" s="4"/>
       <c r="I111" s="4"/>
       <c r="J111" s="1"/>
@@ -4316,14 +4343,14 @@
       <c r="A112" s="9">
         <v>9</v>
       </c>
-      <c r="B112" s="50" t="s">
+      <c r="B112" s="32" t="s">
         <v>66</v>
       </c>
-      <c r="C112" s="29"/>
-      <c r="D112" s="29"/>
-      <c r="E112" s="29"/>
-      <c r="F112" s="29"/>
-      <c r="G112" s="30"/>
+      <c r="C112" s="33"/>
+      <c r="D112" s="33"/>
+      <c r="E112" s="33"/>
+      <c r="F112" s="33"/>
+      <c r="G112" s="34"/>
       <c r="H112" s="4"/>
       <c r="I112" s="4"/>
       <c r="J112" s="1"/>
@@ -4348,14 +4375,14 @@
       <c r="A113" s="9">
         <v>10</v>
       </c>
-      <c r="B113" s="50" t="s">
+      <c r="B113" s="32" t="s">
         <v>67</v>
       </c>
-      <c r="C113" s="29"/>
-      <c r="D113" s="29"/>
-      <c r="E113" s="29"/>
-      <c r="F113" s="29"/>
-      <c r="G113" s="30"/>
+      <c r="C113" s="33"/>
+      <c r="D113" s="33"/>
+      <c r="E113" s="33"/>
+      <c r="F113" s="33"/>
+      <c r="G113" s="34"/>
       <c r="H113" s="4"/>
       <c r="I113" s="4"/>
       <c r="J113" s="1"/>
@@ -4380,14 +4407,14 @@
       <c r="A114" s="9">
         <v>11</v>
       </c>
-      <c r="B114" s="50" t="s">
+      <c r="B114" s="32" t="s">
         <v>68</v>
       </c>
-      <c r="C114" s="29"/>
-      <c r="D114" s="29"/>
-      <c r="E114" s="29"/>
-      <c r="F114" s="29"/>
-      <c r="G114" s="30"/>
+      <c r="C114" s="33"/>
+      <c r="D114" s="33"/>
+      <c r="E114" s="33"/>
+      <c r="F114" s="33"/>
+      <c r="G114" s="34"/>
       <c r="H114" s="4"/>
       <c r="I114" s="4"/>
       <c r="J114" s="1"/>
@@ -4412,14 +4439,14 @@
       <c r="A115" s="9">
         <v>12</v>
       </c>
-      <c r="B115" s="50" t="s">
+      <c r="B115" s="32" t="s">
         <v>69</v>
       </c>
-      <c r="C115" s="29"/>
-      <c r="D115" s="29"/>
-      <c r="E115" s="29"/>
-      <c r="F115" s="29"/>
-      <c r="G115" s="30"/>
+      <c r="C115" s="33"/>
+      <c r="D115" s="33"/>
+      <c r="E115" s="33"/>
+      <c r="F115" s="33"/>
+      <c r="G115" s="34"/>
       <c r="H115" s="4"/>
       <c r="I115" s="4"/>
       <c r="J115" s="1"/>
@@ -4441,17 +4468,17 @@
       <c r="Z115" s="1"/>
     </row>
     <row r="116" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A116" s="32" t="s">
+      <c r="A116" s="31" t="s">
         <v>52</v>
       </c>
-      <c r="B116" s="21"/>
-      <c r="C116" s="21"/>
-      <c r="D116" s="21"/>
-      <c r="E116" s="21"/>
-      <c r="F116" s="21"/>
-      <c r="G116" s="21"/>
-      <c r="H116" s="21"/>
-      <c r="I116" s="22"/>
+      <c r="B116" s="29"/>
+      <c r="C116" s="29"/>
+      <c r="D116" s="29"/>
+      <c r="E116" s="29"/>
+      <c r="F116" s="29"/>
+      <c r="G116" s="29"/>
+      <c r="H116" s="29"/>
+      <c r="I116" s="30"/>
       <c r="J116" s="1"/>
       <c r="K116" s="1"/>
       <c r="L116" s="1"/>
@@ -4471,15 +4498,15 @@
       <c r="Z116" s="1"/>
     </row>
     <row r="117" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A117" s="51"/>
-      <c r="B117" s="21"/>
-      <c r="C117" s="21"/>
-      <c r="D117" s="21"/>
-      <c r="E117" s="21"/>
-      <c r="F117" s="21"/>
-      <c r="G117" s="21"/>
-      <c r="H117" s="21"/>
-      <c r="I117" s="22"/>
+      <c r="A117" s="28"/>
+      <c r="B117" s="29"/>
+      <c r="C117" s="29"/>
+      <c r="D117" s="29"/>
+      <c r="E117" s="29"/>
+      <c r="F117" s="29"/>
+      <c r="G117" s="29"/>
+      <c r="H117" s="29"/>
+      <c r="I117" s="30"/>
       <c r="J117" s="1"/>
       <c r="K117" s="1"/>
       <c r="L117" s="1"/>
@@ -4499,15 +4526,15 @@
       <c r="Z117" s="1"/>
     </row>
     <row r="118" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A118" s="51"/>
-      <c r="B118" s="21"/>
-      <c r="C118" s="21"/>
-      <c r="D118" s="21"/>
-      <c r="E118" s="21"/>
-      <c r="F118" s="21"/>
-      <c r="G118" s="21"/>
-      <c r="H118" s="21"/>
-      <c r="I118" s="22"/>
+      <c r="A118" s="28"/>
+      <c r="B118" s="29"/>
+      <c r="C118" s="29"/>
+      <c r="D118" s="29"/>
+      <c r="E118" s="29"/>
+      <c r="F118" s="29"/>
+      <c r="G118" s="29"/>
+      <c r="H118" s="29"/>
+      <c r="I118" s="30"/>
       <c r="J118" s="1"/>
       <c r="K118" s="1"/>
       <c r="L118" s="1"/>
@@ -4527,15 +4554,15 @@
       <c r="Z118" s="1"/>
     </row>
     <row r="119" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A119" s="51"/>
-      <c r="B119" s="21"/>
-      <c r="C119" s="21"/>
-      <c r="D119" s="21"/>
-      <c r="E119" s="21"/>
-      <c r="F119" s="21"/>
-      <c r="G119" s="21"/>
-      <c r="H119" s="21"/>
-      <c r="I119" s="22"/>
+      <c r="A119" s="28"/>
+      <c r="B119" s="29"/>
+      <c r="C119" s="29"/>
+      <c r="D119" s="29"/>
+      <c r="E119" s="29"/>
+      <c r="F119" s="29"/>
+      <c r="G119" s="29"/>
+      <c r="H119" s="29"/>
+      <c r="I119" s="30"/>
       <c r="J119" s="1"/>
       <c r="K119" s="1"/>
       <c r="L119" s="1"/>
@@ -4555,15 +4582,15 @@
       <c r="Z119" s="1"/>
     </row>
     <row r="120" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A120" s="51"/>
-      <c r="B120" s="21"/>
-      <c r="C120" s="21"/>
-      <c r="D120" s="21"/>
-      <c r="E120" s="21"/>
-      <c r="F120" s="21"/>
-      <c r="G120" s="21"/>
-      <c r="H120" s="21"/>
-      <c r="I120" s="22"/>
+      <c r="A120" s="28"/>
+      <c r="B120" s="29"/>
+      <c r="C120" s="29"/>
+      <c r="D120" s="29"/>
+      <c r="E120" s="29"/>
+      <c r="F120" s="29"/>
+      <c r="G120" s="29"/>
+      <c r="H120" s="29"/>
+      <c r="I120" s="30"/>
       <c r="J120" s="1"/>
       <c r="K120" s="1"/>
       <c r="L120" s="1"/>
@@ -4583,15 +4610,15 @@
       <c r="Z120" s="1"/>
     </row>
     <row r="121" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A121" s="51"/>
-      <c r="B121" s="21"/>
-      <c r="C121" s="21"/>
-      <c r="D121" s="21"/>
-      <c r="E121" s="21"/>
-      <c r="F121" s="21"/>
-      <c r="G121" s="21"/>
-      <c r="H121" s="21"/>
-      <c r="I121" s="22"/>
+      <c r="A121" s="28"/>
+      <c r="B121" s="29"/>
+      <c r="C121" s="29"/>
+      <c r="D121" s="29"/>
+      <c r="E121" s="29"/>
+      <c r="F121" s="29"/>
+      <c r="G121" s="29"/>
+      <c r="H121" s="29"/>
+      <c r="I121" s="30"/>
       <c r="J121" s="1"/>
       <c r="K121" s="1"/>
       <c r="L121" s="1"/>
@@ -4611,17 +4638,17 @@
       <c r="Z121" s="1"/>
     </row>
     <row r="122" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A122" s="32" t="s">
+      <c r="A122" s="31" t="s">
         <v>70</v>
       </c>
-      <c r="B122" s="21"/>
-      <c r="C122" s="21"/>
-      <c r="D122" s="21"/>
-      <c r="E122" s="21"/>
-      <c r="F122" s="21"/>
-      <c r="G122" s="21"/>
-      <c r="H122" s="21"/>
-      <c r="I122" s="22"/>
+      <c r="B122" s="29"/>
+      <c r="C122" s="29"/>
+      <c r="D122" s="29"/>
+      <c r="E122" s="29"/>
+      <c r="F122" s="29"/>
+      <c r="G122" s="29"/>
+      <c r="H122" s="29"/>
+      <c r="I122" s="30"/>
       <c r="J122" s="1"/>
       <c r="K122" s="1"/>
       <c r="L122" s="1"/>
@@ -4641,15 +4668,15 @@
       <c r="Z122" s="1"/>
     </row>
     <row r="123" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A123" s="51"/>
-      <c r="B123" s="21"/>
-      <c r="C123" s="21"/>
-      <c r="D123" s="21"/>
-      <c r="E123" s="21"/>
-      <c r="F123" s="21"/>
-      <c r="G123" s="21"/>
-      <c r="H123" s="21"/>
-      <c r="I123" s="22"/>
+      <c r="A123" s="28"/>
+      <c r="B123" s="29"/>
+      <c r="C123" s="29"/>
+      <c r="D123" s="29"/>
+      <c r="E123" s="29"/>
+      <c r="F123" s="29"/>
+      <c r="G123" s="29"/>
+      <c r="H123" s="29"/>
+      <c r="I123" s="30"/>
       <c r="J123" s="1"/>
       <c r="K123" s="1"/>
       <c r="L123" s="1"/>
@@ -4669,15 +4696,15 @@
       <c r="Z123" s="1"/>
     </row>
     <row r="124" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A124" s="51"/>
-      <c r="B124" s="21"/>
-      <c r="C124" s="21"/>
-      <c r="D124" s="21"/>
-      <c r="E124" s="21"/>
-      <c r="F124" s="21"/>
-      <c r="G124" s="21"/>
-      <c r="H124" s="21"/>
-      <c r="I124" s="22"/>
+      <c r="A124" s="28"/>
+      <c r="B124" s="29"/>
+      <c r="C124" s="29"/>
+      <c r="D124" s="29"/>
+      <c r="E124" s="29"/>
+      <c r="F124" s="29"/>
+      <c r="G124" s="29"/>
+      <c r="H124" s="29"/>
+      <c r="I124" s="30"/>
       <c r="J124" s="1"/>
       <c r="K124" s="1"/>
       <c r="L124" s="1"/>
@@ -4697,15 +4724,15 @@
       <c r="Z124" s="1"/>
     </row>
     <row r="125" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A125" s="51"/>
-      <c r="B125" s="21"/>
-      <c r="C125" s="21"/>
-      <c r="D125" s="21"/>
-      <c r="E125" s="21"/>
-      <c r="F125" s="21"/>
-      <c r="G125" s="21"/>
-      <c r="H125" s="21"/>
-      <c r="I125" s="22"/>
+      <c r="A125" s="28"/>
+      <c r="B125" s="29"/>
+      <c r="C125" s="29"/>
+      <c r="D125" s="29"/>
+      <c r="E125" s="29"/>
+      <c r="F125" s="29"/>
+      <c r="G125" s="29"/>
+      <c r="H125" s="29"/>
+      <c r="I125" s="30"/>
       <c r="J125" s="1"/>
       <c r="K125" s="1"/>
       <c r="L125" s="1"/>
@@ -4725,15 +4752,15 @@
       <c r="Z125" s="1"/>
     </row>
     <row r="126" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A126" s="51"/>
-      <c r="B126" s="21"/>
-      <c r="C126" s="21"/>
-      <c r="D126" s="21"/>
-      <c r="E126" s="21"/>
-      <c r="F126" s="21"/>
-      <c r="G126" s="21"/>
-      <c r="H126" s="21"/>
-      <c r="I126" s="22"/>
+      <c r="A126" s="28"/>
+      <c r="B126" s="29"/>
+      <c r="C126" s="29"/>
+      <c r="D126" s="29"/>
+      <c r="E126" s="29"/>
+      <c r="F126" s="29"/>
+      <c r="G126" s="29"/>
+      <c r="H126" s="29"/>
+      <c r="I126" s="30"/>
       <c r="J126" s="1"/>
       <c r="K126" s="1"/>
       <c r="L126" s="1"/>
@@ -4753,15 +4780,15 @@
       <c r="Z126" s="1"/>
     </row>
     <row r="127" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A127" s="51"/>
-      <c r="B127" s="21"/>
-      <c r="C127" s="21"/>
-      <c r="D127" s="21"/>
-      <c r="E127" s="21"/>
-      <c r="F127" s="21"/>
-      <c r="G127" s="21"/>
-      <c r="H127" s="21"/>
-      <c r="I127" s="22"/>
+      <c r="A127" s="28"/>
+      <c r="B127" s="29"/>
+      <c r="C127" s="29"/>
+      <c r="D127" s="29"/>
+      <c r="E127" s="29"/>
+      <c r="F127" s="29"/>
+      <c r="G127" s="29"/>
+      <c r="H127" s="29"/>
+      <c r="I127" s="30"/>
       <c r="J127" s="1"/>
       <c r="K127" s="1"/>
       <c r="L127" s="1"/>
@@ -4781,17 +4808,17 @@
       <c r="Z127" s="1"/>
     </row>
     <row r="128" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A128" s="32" t="s">
+      <c r="A128" s="31" t="s">
         <v>71</v>
       </c>
-      <c r="B128" s="21"/>
-      <c r="C128" s="21"/>
-      <c r="D128" s="21"/>
-      <c r="E128" s="21"/>
-      <c r="F128" s="21"/>
-      <c r="G128" s="21"/>
-      <c r="H128" s="21"/>
-      <c r="I128" s="22"/>
+      <c r="B128" s="29"/>
+      <c r="C128" s="29"/>
+      <c r="D128" s="29"/>
+      <c r="E128" s="29"/>
+      <c r="F128" s="29"/>
+      <c r="G128" s="29"/>
+      <c r="H128" s="29"/>
+      <c r="I128" s="30"/>
       <c r="J128" s="1"/>
       <c r="K128" s="1"/>
       <c r="L128" s="1"/>
@@ -4811,15 +4838,15 @@
       <c r="Z128" s="1"/>
     </row>
     <row r="129" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A129" s="51"/>
-      <c r="B129" s="21"/>
-      <c r="C129" s="21"/>
-      <c r="D129" s="21"/>
-      <c r="E129" s="21"/>
-      <c r="F129" s="21"/>
-      <c r="G129" s="21"/>
-      <c r="H129" s="21"/>
-      <c r="I129" s="22"/>
+      <c r="A129" s="28"/>
+      <c r="B129" s="29"/>
+      <c r="C129" s="29"/>
+      <c r="D129" s="29"/>
+      <c r="E129" s="29"/>
+      <c r="F129" s="29"/>
+      <c r="G129" s="29"/>
+      <c r="H129" s="29"/>
+      <c r="I129" s="30"/>
       <c r="J129" s="1"/>
       <c r="K129" s="1"/>
       <c r="L129" s="1"/>
@@ -4839,15 +4866,15 @@
       <c r="Z129" s="1"/>
     </row>
     <row r="130" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A130" s="51"/>
-      <c r="B130" s="21"/>
-      <c r="C130" s="21"/>
-      <c r="D130" s="21"/>
-      <c r="E130" s="21"/>
-      <c r="F130" s="21"/>
-      <c r="G130" s="21"/>
-      <c r="H130" s="21"/>
-      <c r="I130" s="22"/>
+      <c r="A130" s="28"/>
+      <c r="B130" s="29"/>
+      <c r="C130" s="29"/>
+      <c r="D130" s="29"/>
+      <c r="E130" s="29"/>
+      <c r="F130" s="29"/>
+      <c r="G130" s="29"/>
+      <c r="H130" s="29"/>
+      <c r="I130" s="30"/>
       <c r="J130" s="1"/>
       <c r="K130" s="1"/>
       <c r="L130" s="1"/>
@@ -4867,15 +4894,15 @@
       <c r="Z130" s="1"/>
     </row>
     <row r="131" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A131" s="51"/>
-      <c r="B131" s="21"/>
-      <c r="C131" s="21"/>
-      <c r="D131" s="21"/>
-      <c r="E131" s="21"/>
-      <c r="F131" s="21"/>
-      <c r="G131" s="21"/>
-      <c r="H131" s="21"/>
-      <c r="I131" s="22"/>
+      <c r="A131" s="28"/>
+      <c r="B131" s="29"/>
+      <c r="C131" s="29"/>
+      <c r="D131" s="29"/>
+      <c r="E131" s="29"/>
+      <c r="F131" s="29"/>
+      <c r="G131" s="29"/>
+      <c r="H131" s="29"/>
+      <c r="I131" s="30"/>
       <c r="J131" s="1"/>
       <c r="K131" s="1"/>
       <c r="L131" s="1"/>
@@ -4895,15 +4922,15 @@
       <c r="Z131" s="1"/>
     </row>
     <row r="132" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A132" s="18"/>
-      <c r="B132" s="16"/>
-      <c r="C132" s="16"/>
-      <c r="D132" s="16"/>
-      <c r="E132" s="16"/>
-      <c r="F132" s="16"/>
-      <c r="G132" s="16"/>
-      <c r="H132" s="16"/>
-      <c r="I132" s="17"/>
+      <c r="A132" s="28"/>
+      <c r="B132" s="29"/>
+      <c r="C132" s="29"/>
+      <c r="D132" s="29"/>
+      <c r="E132" s="29"/>
+      <c r="F132" s="29"/>
+      <c r="G132" s="29"/>
+      <c r="H132" s="29"/>
+      <c r="I132" s="30"/>
       <c r="J132" s="1"/>
       <c r="K132" s="1"/>
       <c r="L132" s="1"/>
@@ -4922,33 +4949,33 @@
       <c r="Y132" s="1"/>
       <c r="Z132" s="1"/>
     </row>
-    <row r="133" spans="1:26" s="83" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A133" s="80"/>
-      <c r="B133" s="81"/>
-      <c r="C133" s="81"/>
-      <c r="D133" s="81"/>
-      <c r="E133" s="81"/>
-      <c r="F133" s="81"/>
-      <c r="G133" s="81"/>
-      <c r="H133" s="81"/>
-      <c r="I133" s="81"/>
-      <c r="J133" s="82"/>
-      <c r="K133" s="82"/>
-      <c r="L133" s="82"/>
-      <c r="M133" s="82"/>
-      <c r="N133" s="82"/>
-      <c r="O133" s="82"/>
-      <c r="P133" s="82"/>
-      <c r="Q133" s="82"/>
-      <c r="R133" s="82"/>
-      <c r="S133" s="82"/>
-      <c r="T133" s="82"/>
-      <c r="U133" s="82"/>
-      <c r="V133" s="82"/>
-      <c r="W133" s="82"/>
-      <c r="X133" s="82"/>
-      <c r="Y133" s="82"/>
-      <c r="Z133" s="82"/>
+    <row r="133" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A133" s="77"/>
+      <c r="B133" s="78"/>
+      <c r="C133" s="78"/>
+      <c r="D133" s="78"/>
+      <c r="E133" s="78"/>
+      <c r="F133" s="78"/>
+      <c r="G133" s="78"/>
+      <c r="H133" s="78"/>
+      <c r="I133" s="79"/>
+      <c r="J133" s="1"/>
+      <c r="K133" s="1"/>
+      <c r="L133" s="1"/>
+      <c r="M133" s="1"/>
+      <c r="N133" s="1"/>
+      <c r="O133" s="1"/>
+      <c r="P133" s="1"/>
+      <c r="Q133" s="1"/>
+      <c r="R133" s="1"/>
+      <c r="S133" s="1"/>
+      <c r="T133" s="1"/>
+      <c r="U133" s="1"/>
+      <c r="V133" s="1"/>
+      <c r="W133" s="1"/>
+      <c r="X133" s="1"/>
+      <c r="Y133" s="1"/>
+      <c r="Z133" s="1"/>
     </row>
     <row r="134" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A134" s="1"/>
@@ -10998,69 +11025,41 @@
       <c r="Y349" s="1"/>
       <c r="Z349" s="1"/>
     </row>
-    <row r="350" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A350" s="1"/>
-      <c r="B350" s="1"/>
-      <c r="C350" s="1"/>
-      <c r="D350" s="1"/>
-      <c r="E350" s="1"/>
-      <c r="F350" s="1"/>
-      <c r="G350" s="1"/>
-      <c r="H350" s="1"/>
-      <c r="I350" s="1"/>
-      <c r="J350" s="1"/>
-      <c r="K350" s="1"/>
-      <c r="L350" s="1"/>
-      <c r="M350" s="1"/>
-      <c r="N350" s="1"/>
-      <c r="O350" s="1"/>
-      <c r="P350" s="1"/>
-      <c r="Q350" s="1"/>
-      <c r="R350" s="1"/>
-      <c r="S350" s="1"/>
-      <c r="T350" s="1"/>
-      <c r="U350" s="1"/>
-      <c r="V350" s="1"/>
-      <c r="W350" s="1"/>
-      <c r="X350" s="1"/>
-      <c r="Y350" s="1"/>
-      <c r="Z350" s="1"/>
-    </row>
   </sheetData>
-  <mergeCells count="80">
-    <mergeCell ref="D8:I9"/>
-    <mergeCell ref="A120:I120"/>
-    <mergeCell ref="A119:I119"/>
-    <mergeCell ref="A118:I118"/>
-    <mergeCell ref="A117:I117"/>
-    <mergeCell ref="A129:I129"/>
+  <mergeCells count="81">
+    <mergeCell ref="A132:I132"/>
     <mergeCell ref="A133:I133"/>
-    <mergeCell ref="A122:I122"/>
-    <mergeCell ref="A123:I123"/>
-    <mergeCell ref="A126:I126"/>
-    <mergeCell ref="A127:I127"/>
-    <mergeCell ref="A128:I128"/>
-    <mergeCell ref="A124:I124"/>
-    <mergeCell ref="A125:I125"/>
-    <mergeCell ref="A130:I130"/>
-    <mergeCell ref="A131:I131"/>
-    <mergeCell ref="B113:G113"/>
-    <mergeCell ref="B114:G114"/>
-    <mergeCell ref="B115:G115"/>
-    <mergeCell ref="A116:I116"/>
-    <mergeCell ref="A121:I121"/>
-    <mergeCell ref="B108:G108"/>
-    <mergeCell ref="B109:G109"/>
-    <mergeCell ref="B110:G110"/>
-    <mergeCell ref="B111:G111"/>
-    <mergeCell ref="B112:G112"/>
-    <mergeCell ref="B103:G103"/>
-    <mergeCell ref="B104:G104"/>
-    <mergeCell ref="B105:G105"/>
-    <mergeCell ref="B106:G106"/>
-    <mergeCell ref="B107:G107"/>
-    <mergeCell ref="B100:C100"/>
-    <mergeCell ref="E100:I101"/>
+    <mergeCell ref="A8:B8"/>
+    <mergeCell ref="A9:B9"/>
+    <mergeCell ref="C8:C9"/>
+    <mergeCell ref="A1:I2"/>
+    <mergeCell ref="A3:I3"/>
+    <mergeCell ref="A4:I4"/>
+    <mergeCell ref="E6:F6"/>
+    <mergeCell ref="E7:F7"/>
+    <mergeCell ref="A5:I5"/>
+    <mergeCell ref="C6:D6"/>
+    <mergeCell ref="C7:D7"/>
+    <mergeCell ref="A6:B6"/>
+    <mergeCell ref="A7:B7"/>
+    <mergeCell ref="A26:I26"/>
+    <mergeCell ref="A47:C47"/>
+    <mergeCell ref="D47:F47"/>
+    <mergeCell ref="G47:I47"/>
+    <mergeCell ref="A10:D10"/>
+    <mergeCell ref="F10:I10"/>
+    <mergeCell ref="E11:E25"/>
+    <mergeCell ref="A24:B24"/>
+    <mergeCell ref="C24:D25"/>
+    <mergeCell ref="F24:G24"/>
+    <mergeCell ref="H24:I25"/>
+    <mergeCell ref="A25:B25"/>
+    <mergeCell ref="F25:G25"/>
+    <mergeCell ref="G98:I98"/>
+    <mergeCell ref="G99:I99"/>
+    <mergeCell ref="A68:C68"/>
+    <mergeCell ref="D68:F68"/>
+    <mergeCell ref="G68:I68"/>
     <mergeCell ref="A101:C101"/>
     <mergeCell ref="D100:D101"/>
     <mergeCell ref="A102:I102"/>
@@ -11077,40 +11076,41 @@
     <mergeCell ref="G95:I95"/>
     <mergeCell ref="G96:I96"/>
     <mergeCell ref="G97:I97"/>
-    <mergeCell ref="G98:I98"/>
-    <mergeCell ref="G99:I99"/>
-    <mergeCell ref="A68:C68"/>
-    <mergeCell ref="D68:F68"/>
-    <mergeCell ref="G68:I68"/>
-    <mergeCell ref="A26:I26"/>
-    <mergeCell ref="A47:C47"/>
-    <mergeCell ref="D47:F47"/>
-    <mergeCell ref="G47:I47"/>
-    <mergeCell ref="A10:D10"/>
-    <mergeCell ref="F10:I10"/>
-    <mergeCell ref="E11:E25"/>
-    <mergeCell ref="A24:B24"/>
-    <mergeCell ref="C24:D25"/>
-    <mergeCell ref="F24:G24"/>
-    <mergeCell ref="H24:I25"/>
-    <mergeCell ref="A25:B25"/>
-    <mergeCell ref="F25:G25"/>
-    <mergeCell ref="A4:I4"/>
-    <mergeCell ref="E6:F6"/>
-    <mergeCell ref="E7:F7"/>
-    <mergeCell ref="A5:I5"/>
-    <mergeCell ref="C6:D6"/>
-    <mergeCell ref="C7:D7"/>
-    <mergeCell ref="A6:B6"/>
-    <mergeCell ref="A7:B7"/>
-    <mergeCell ref="A8:B8"/>
-    <mergeCell ref="A9:B9"/>
-    <mergeCell ref="C8:C9"/>
-    <mergeCell ref="A1:I2"/>
-    <mergeCell ref="A3:I3"/>
+    <mergeCell ref="A121:I121"/>
+    <mergeCell ref="B108:G108"/>
+    <mergeCell ref="B109:G109"/>
+    <mergeCell ref="B110:G110"/>
+    <mergeCell ref="B111:G111"/>
+    <mergeCell ref="B112:G112"/>
+    <mergeCell ref="A129:I129"/>
+    <mergeCell ref="A122:I122"/>
+    <mergeCell ref="A123:I123"/>
+    <mergeCell ref="A126:I126"/>
+    <mergeCell ref="A127:I127"/>
+    <mergeCell ref="A128:I128"/>
+    <mergeCell ref="A124:I124"/>
+    <mergeCell ref="A125:I125"/>
+    <mergeCell ref="A130:I130"/>
+    <mergeCell ref="A131:I131"/>
+    <mergeCell ref="D8:I9"/>
+    <mergeCell ref="A120:I120"/>
+    <mergeCell ref="A119:I119"/>
+    <mergeCell ref="A118:I118"/>
+    <mergeCell ref="A117:I117"/>
+    <mergeCell ref="B113:G113"/>
+    <mergeCell ref="B114:G114"/>
+    <mergeCell ref="B115:G115"/>
+    <mergeCell ref="A116:I116"/>
+    <mergeCell ref="B103:G103"/>
+    <mergeCell ref="B104:G104"/>
+    <mergeCell ref="B105:G105"/>
+    <mergeCell ref="B106:G106"/>
+    <mergeCell ref="B107:G107"/>
+    <mergeCell ref="B100:C100"/>
+    <mergeCell ref="E100:I101"/>
   </mergeCells>
   <printOptions horizontalCentered="1" gridLines="1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0" footer="0"/>
-  <pageSetup paperSize="14" pageOrder="overThenDown" orientation="portrait" cellComments="atEnd"/>
+  <pageSetup paperSize="14" pageOrder="overThenDown" orientation="portrait" cellComments="atEnd" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
informes de equipo general y mantto variador agregados
</commit_message>
<xml_diff>
--- a/public/informes-templates/INFORME VARIADOR REPARACION.xlsx
+++ b/public/informes-templates/INFORME VARIADOR REPARACION.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30326"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{02C4A046-F2A7-472F-A6F8-996D3E80A366}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{260FD4E6-13B0-4F64-B968-042B8B5E456A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -321,10 +321,11 @@
       <name val="Calibri"/>
     </font>
     <font>
+      <i/>
       <sz val="12"/>
       <color theme="1"/>
-      <name val="Times New Roman"/>
-      <family val="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="6">
@@ -592,7 +593,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="80">
+  <cellXfs count="78">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -672,9 +673,6 @@
     <xf numFmtId="49" fontId="5" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="12" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
@@ -684,41 +682,38 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="12" fillId="4" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="12" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
@@ -726,22 +721,46 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="49" fontId="5" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="9" fillId="3" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="9" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -762,74 +781,50 @@
     <xf numFmtId="0" fontId="4" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="5" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="9" fillId="3" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="12" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="4" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1056,17 +1051,17 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:26" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="73" t="s">
+      <c r="A1" s="39" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="29"/>
-      <c r="C1" s="29"/>
-      <c r="D1" s="29"/>
-      <c r="E1" s="29"/>
-      <c r="F1" s="29"/>
-      <c r="G1" s="29"/>
-      <c r="H1" s="29"/>
-      <c r="I1" s="30"/>
+      <c r="B1" s="28"/>
+      <c r="C1" s="28"/>
+      <c r="D1" s="28"/>
+      <c r="E1" s="28"/>
+      <c r="F1" s="28"/>
+      <c r="G1" s="28"/>
+      <c r="H1" s="28"/>
+      <c r="I1" s="29"/>
       <c r="J1" s="1"/>
       <c r="K1" s="1"/>
       <c r="L1" s="1"/>
@@ -1086,15 +1081,15 @@
       <c r="Z1" s="1"/>
     </row>
     <row r="2" spans="1:26" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="58"/>
-      <c r="B2" s="43"/>
-      <c r="C2" s="43"/>
-      <c r="D2" s="43"/>
-      <c r="E2" s="43"/>
-      <c r="F2" s="43"/>
-      <c r="G2" s="43"/>
-      <c r="H2" s="43"/>
-      <c r="I2" s="44"/>
+      <c r="A2" s="40"/>
+      <c r="B2" s="41"/>
+      <c r="C2" s="41"/>
+      <c r="D2" s="41"/>
+      <c r="E2" s="41"/>
+      <c r="F2" s="41"/>
+      <c r="G2" s="41"/>
+      <c r="H2" s="41"/>
+      <c r="I2" s="42"/>
       <c r="J2" s="1"/>
       <c r="K2" s="1"/>
       <c r="L2" s="1"/>
@@ -1114,15 +1109,15 @@
       <c r="Z2" s="1"/>
     </row>
     <row r="3" spans="1:26" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="74"/>
-      <c r="B3" s="75"/>
-      <c r="C3" s="75"/>
-      <c r="D3" s="75"/>
-      <c r="E3" s="75"/>
-      <c r="F3" s="75"/>
-      <c r="G3" s="75"/>
-      <c r="H3" s="75"/>
-      <c r="I3" s="76"/>
+      <c r="A3" s="77"/>
+      <c r="B3" s="77"/>
+      <c r="C3" s="77"/>
+      <c r="D3" s="77"/>
+      <c r="E3" s="77"/>
+      <c r="F3" s="77"/>
+      <c r="G3" s="77"/>
+      <c r="H3" s="77"/>
+      <c r="I3" s="77"/>
       <c r="J3" s="1"/>
       <c r="K3" s="1"/>
       <c r="L3" s="1"/>
@@ -1142,15 +1137,15 @@
       <c r="Z3" s="1"/>
     </row>
     <row r="4" spans="1:26" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="60"/>
-      <c r="B4" s="43"/>
-      <c r="C4" s="43"/>
-      <c r="D4" s="43"/>
-      <c r="E4" s="43"/>
-      <c r="F4" s="43"/>
-      <c r="G4" s="43"/>
-      <c r="H4" s="43"/>
-      <c r="I4" s="43"/>
+      <c r="A4" s="43"/>
+      <c r="B4" s="41"/>
+      <c r="C4" s="41"/>
+      <c r="D4" s="41"/>
+      <c r="E4" s="41"/>
+      <c r="F4" s="41"/>
+      <c r="G4" s="41"/>
+      <c r="H4" s="41"/>
+      <c r="I4" s="41"/>
       <c r="J4" s="1"/>
       <c r="K4" s="1"/>
       <c r="L4" s="1"/>
@@ -1170,17 +1165,17 @@
       <c r="Z4" s="1"/>
     </row>
     <row r="5" spans="1:26" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="57" t="s">
+      <c r="A5" s="37" t="s">
         <v>2</v>
       </c>
-      <c r="B5" s="62"/>
-      <c r="C5" s="62"/>
-      <c r="D5" s="62"/>
-      <c r="E5" s="62"/>
-      <c r="F5" s="62"/>
-      <c r="G5" s="62"/>
-      <c r="H5" s="62"/>
-      <c r="I5" s="63"/>
+      <c r="B5" s="47"/>
+      <c r="C5" s="47"/>
+      <c r="D5" s="47"/>
+      <c r="E5" s="47"/>
+      <c r="F5" s="47"/>
+      <c r="G5" s="47"/>
+      <c r="H5" s="47"/>
+      <c r="I5" s="48"/>
       <c r="J5" s="1"/>
       <c r="K5" s="1"/>
       <c r="L5" s="1"/>
@@ -1200,18 +1195,18 @@
       <c r="Z5" s="1"/>
     </row>
     <row r="6" spans="1:26" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="64" t="s">
+      <c r="A6" s="33" t="s">
         <v>3</v>
       </c>
-      <c r="B6" s="65"/>
-      <c r="C6" s="64" t="s">
+      <c r="B6" s="34"/>
+      <c r="C6" s="33" t="s">
         <v>4</v>
       </c>
-      <c r="D6" s="65"/>
-      <c r="E6" s="35" t="s">
+      <c r="D6" s="34"/>
+      <c r="E6" s="44" t="s">
         <v>5</v>
       </c>
-      <c r="F6" s="34"/>
+      <c r="F6" s="45"/>
       <c r="G6" s="3" t="s">
         <v>6</v>
       </c>
@@ -1240,12 +1235,12 @@
       <c r="Z6" s="1"/>
     </row>
     <row r="7" spans="1:26" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="68"/>
-      <c r="B7" s="69"/>
-      <c r="C7" s="66"/>
-      <c r="D7" s="67"/>
-      <c r="E7" s="61"/>
-      <c r="F7" s="30"/>
+      <c r="A7" s="51"/>
+      <c r="B7" s="52"/>
+      <c r="C7" s="49"/>
+      <c r="D7" s="50"/>
+      <c r="E7" s="46"/>
+      <c r="F7" s="29"/>
       <c r="G7" s="16"/>
       <c r="H7" s="16"/>
       <c r="I7" s="16"/>
@@ -1268,19 +1263,19 @@
       <c r="Z7" s="1"/>
     </row>
     <row r="8" spans="1:26" x14ac:dyDescent="0.25">
-      <c r="A8" s="64" t="s">
+      <c r="A8" s="33" t="s">
         <v>9</v>
       </c>
-      <c r="B8" s="65"/>
-      <c r="C8" s="57" t="s">
+      <c r="B8" s="34"/>
+      <c r="C8" s="37" t="s">
         <v>10</v>
       </c>
-      <c r="D8" s="27"/>
-      <c r="E8" s="27"/>
-      <c r="F8" s="27"/>
-      <c r="G8" s="27"/>
-      <c r="H8" s="27"/>
-      <c r="I8" s="27"/>
+      <c r="D8" s="75"/>
+      <c r="E8" s="75"/>
+      <c r="F8" s="75"/>
+      <c r="G8" s="75"/>
+      <c r="H8" s="75"/>
+      <c r="I8" s="75"/>
       <c r="J8" s="1"/>
       <c r="K8" s="1"/>
       <c r="L8" s="1"/>
@@ -1300,15 +1295,15 @@
       <c r="Z8" s="1"/>
     </row>
     <row r="9" spans="1:26" x14ac:dyDescent="0.25">
-      <c r="A9" s="70"/>
-      <c r="B9" s="71"/>
-      <c r="C9" s="72"/>
-      <c r="D9" s="27"/>
-      <c r="E9" s="27"/>
-      <c r="F9" s="27"/>
-      <c r="G9" s="27"/>
-      <c r="H9" s="27"/>
-      <c r="I9" s="27"/>
+      <c r="A9" s="35"/>
+      <c r="B9" s="36"/>
+      <c r="C9" s="38"/>
+      <c r="D9" s="75"/>
+      <c r="E9" s="75"/>
+      <c r="F9" s="75"/>
+      <c r="G9" s="75"/>
+      <c r="H9" s="75"/>
+      <c r="I9" s="75"/>
       <c r="J9" s="1"/>
       <c r="K9" s="1"/>
       <c r="L9" s="1"/>
@@ -1328,19 +1323,19 @@
       <c r="Z9" s="1"/>
     </row>
     <row r="10" spans="1:26" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="31" t="s">
+      <c r="A10" s="56" t="s">
         <v>11</v>
       </c>
-      <c r="B10" s="29"/>
-      <c r="C10" s="29"/>
-      <c r="D10" s="51"/>
+      <c r="B10" s="28"/>
+      <c r="C10" s="28"/>
+      <c r="D10" s="57"/>
       <c r="E10" s="5"/>
-      <c r="F10" s="52" t="s">
+      <c r="F10" s="58" t="s">
         <v>12</v>
       </c>
-      <c r="G10" s="51"/>
-      <c r="H10" s="51"/>
-      <c r="I10" s="51"/>
+      <c r="G10" s="57"/>
+      <c r="H10" s="57"/>
+      <c r="I10" s="57"/>
       <c r="J10" s="1"/>
       <c r="K10" s="1"/>
       <c r="L10" s="1"/>
@@ -1366,7 +1361,7 @@
       <c r="B11" s="6"/>
       <c r="C11" s="10"/>
       <c r="D11" s="11"/>
-      <c r="E11" s="53"/>
+      <c r="E11" s="59"/>
       <c r="F11" s="2" t="s">
         <v>13</v>
       </c>
@@ -1398,7 +1393,7 @@
       <c r="B12" s="6"/>
       <c r="C12" s="12"/>
       <c r="D12" s="13"/>
-      <c r="E12" s="54"/>
+      <c r="E12" s="60"/>
       <c r="F12" s="2" t="s">
         <v>14</v>
       </c>
@@ -1430,7 +1425,7 @@
       <c r="B13" s="6"/>
       <c r="C13" s="12"/>
       <c r="D13" s="13"/>
-      <c r="E13" s="54"/>
+      <c r="E13" s="60"/>
       <c r="F13" s="2" t="s">
         <v>15</v>
       </c>
@@ -1462,7 +1457,7 @@
       <c r="B14" s="4"/>
       <c r="C14" s="12"/>
       <c r="D14" s="13"/>
-      <c r="E14" s="54"/>
+      <c r="E14" s="60"/>
       <c r="F14" s="2" t="s">
         <v>16</v>
       </c>
@@ -1494,7 +1489,7 @@
       <c r="B15" s="6"/>
       <c r="C15" s="12"/>
       <c r="D15" s="13"/>
-      <c r="E15" s="54"/>
+      <c r="E15" s="60"/>
       <c r="F15" s="2" t="s">
         <v>17</v>
       </c>
@@ -1526,7 +1521,7 @@
       <c r="B16" s="4"/>
       <c r="C16" s="12"/>
       <c r="D16" s="13"/>
-      <c r="E16" s="54"/>
+      <c r="E16" s="60"/>
       <c r="F16" s="2" t="s">
         <v>18</v>
       </c>
@@ -1558,7 +1553,7 @@
       <c r="B17" s="4"/>
       <c r="C17" s="12"/>
       <c r="D17" s="13"/>
-      <c r="E17" s="54"/>
+      <c r="E17" s="60"/>
       <c r="F17" s="2" t="s">
         <v>19</v>
       </c>
@@ -1590,7 +1585,7 @@
       <c r="B18" s="4"/>
       <c r="C18" s="12"/>
       <c r="D18" s="13"/>
-      <c r="E18" s="54"/>
+      <c r="E18" s="60"/>
       <c r="F18" s="2" t="s">
         <v>20</v>
       </c>
@@ -1622,7 +1617,7 @@
       <c r="B19" s="4"/>
       <c r="C19" s="12"/>
       <c r="D19" s="13"/>
-      <c r="E19" s="54"/>
+      <c r="E19" s="60"/>
       <c r="F19" s="2" t="s">
         <v>21</v>
       </c>
@@ -1654,7 +1649,7 @@
       <c r="B20" s="4"/>
       <c r="C20" s="12"/>
       <c r="D20" s="13"/>
-      <c r="E20" s="54"/>
+      <c r="E20" s="60"/>
       <c r="F20" s="2" t="s">
         <v>22</v>
       </c>
@@ -1686,7 +1681,7 @@
       <c r="B21" s="4"/>
       <c r="C21" s="12"/>
       <c r="D21" s="13"/>
-      <c r="E21" s="54"/>
+      <c r="E21" s="60"/>
       <c r="F21" s="2" t="s">
         <v>23</v>
       </c>
@@ -1718,7 +1713,7 @@
       <c r="B22" s="4"/>
       <c r="C22" s="12"/>
       <c r="D22" s="13"/>
-      <c r="E22" s="54"/>
+      <c r="E22" s="60"/>
       <c r="F22" s="2" t="s">
         <v>24</v>
       </c>
@@ -1750,7 +1745,7 @@
       <c r="B23" s="4"/>
       <c r="C23" s="14"/>
       <c r="D23" s="15"/>
-      <c r="E23" s="54"/>
+      <c r="E23" s="60"/>
       <c r="F23" s="2" t="s">
         <v>25</v>
       </c>
@@ -1776,23 +1771,23 @@
       <c r="Z23" s="1"/>
     </row>
     <row r="24" spans="1:26" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="56" t="s">
+      <c r="A24" s="62" t="s">
         <v>26</v>
       </c>
-      <c r="B24" s="34"/>
-      <c r="C24" s="57" t="s">
+      <c r="B24" s="45"/>
+      <c r="C24" s="37" t="s">
         <v>27</v>
       </c>
-      <c r="D24" s="30"/>
-      <c r="E24" s="54"/>
-      <c r="F24" s="56" t="s">
+      <c r="D24" s="29"/>
+      <c r="E24" s="60"/>
+      <c r="F24" s="62" t="s">
         <v>26</v>
       </c>
-      <c r="G24" s="34"/>
-      <c r="H24" s="57" t="s">
+      <c r="G24" s="45"/>
+      <c r="H24" s="37" t="s">
         <v>28</v>
       </c>
-      <c r="I24" s="30"/>
+      <c r="I24" s="29"/>
       <c r="J24" s="1"/>
       <c r="K24" s="1"/>
       <c r="L24" s="1"/>
@@ -1812,15 +1807,15 @@
       <c r="Z24" s="1"/>
     </row>
     <row r="25" spans="1:26" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="59"/>
-      <c r="B25" s="44"/>
-      <c r="C25" s="58"/>
-      <c r="D25" s="44"/>
-      <c r="E25" s="55"/>
-      <c r="F25" s="59"/>
-      <c r="G25" s="44"/>
-      <c r="H25" s="58"/>
-      <c r="I25" s="44"/>
+      <c r="A25" s="63"/>
+      <c r="B25" s="42"/>
+      <c r="C25" s="40"/>
+      <c r="D25" s="42"/>
+      <c r="E25" s="61"/>
+      <c r="F25" s="63"/>
+      <c r="G25" s="42"/>
+      <c r="H25" s="40"/>
+      <c r="I25" s="42"/>
       <c r="J25" s="1"/>
       <c r="K25" s="1"/>
       <c r="L25" s="1"/>
@@ -1840,17 +1835,17 @@
       <c r="Z25" s="1"/>
     </row>
     <row r="26" spans="1:26" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="50" t="s">
+      <c r="A26" s="53" t="s">
         <v>29</v>
       </c>
-      <c r="B26" s="33"/>
-      <c r="C26" s="33"/>
-      <c r="D26" s="33"/>
-      <c r="E26" s="33"/>
-      <c r="F26" s="33"/>
-      <c r="G26" s="33"/>
-      <c r="H26" s="33"/>
-      <c r="I26" s="34"/>
+      <c r="B26" s="54"/>
+      <c r="C26" s="54"/>
+      <c r="D26" s="54"/>
+      <c r="E26" s="54"/>
+      <c r="F26" s="54"/>
+      <c r="G26" s="54"/>
+      <c r="H26" s="54"/>
+      <c r="I26" s="45"/>
       <c r="J26" s="1"/>
       <c r="K26" s="1"/>
       <c r="L26" s="1"/>
@@ -2430,21 +2425,21 @@
       <c r="Z46" s="1"/>
     </row>
     <row r="47" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A47" s="40" t="s">
+      <c r="A47" s="55" t="s">
         <v>30</v>
       </c>
-      <c r="B47" s="33"/>
-      <c r="C47" s="34"/>
-      <c r="D47" s="40" t="s">
+      <c r="B47" s="54"/>
+      <c r="C47" s="45"/>
+      <c r="D47" s="55" t="s">
         <v>31</v>
       </c>
-      <c r="E47" s="33"/>
-      <c r="F47" s="34"/>
-      <c r="G47" s="40" t="s">
+      <c r="E47" s="54"/>
+      <c r="F47" s="45"/>
+      <c r="G47" s="55" t="s">
         <v>32</v>
       </c>
-      <c r="H47" s="33"/>
-      <c r="I47" s="34"/>
+      <c r="H47" s="54"/>
+      <c r="I47" s="45"/>
       <c r="J47" s="1"/>
       <c r="K47" s="1"/>
       <c r="L47" s="1"/>
@@ -3024,21 +3019,21 @@
       <c r="Z67" s="1"/>
     </row>
     <row r="68" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A68" s="40" t="s">
+      <c r="A68" s="55" t="s">
         <v>33</v>
       </c>
-      <c r="B68" s="33"/>
-      <c r="C68" s="34"/>
-      <c r="D68" s="40" t="s">
+      <c r="B68" s="54"/>
+      <c r="C68" s="45"/>
+      <c r="D68" s="55" t="s">
         <v>34</v>
       </c>
-      <c r="E68" s="33"/>
-      <c r="F68" s="34"/>
-      <c r="G68" s="49" t="s">
+      <c r="E68" s="54"/>
+      <c r="F68" s="45"/>
+      <c r="G68" s="65" t="s">
         <v>35</v>
       </c>
-      <c r="H68" s="33"/>
-      <c r="I68" s="34"/>
+      <c r="H68" s="54"/>
+      <c r="I68" s="45"/>
       <c r="J68" s="1"/>
       <c r="K68" s="1"/>
       <c r="L68" s="1"/>
@@ -3618,21 +3613,21 @@
       <c r="Z88" s="1"/>
     </row>
     <row r="89" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A89" s="40" t="s">
+      <c r="A89" s="55" t="s">
         <v>36</v>
       </c>
-      <c r="B89" s="33"/>
-      <c r="C89" s="34"/>
-      <c r="D89" s="40" t="s">
+      <c r="B89" s="54"/>
+      <c r="C89" s="45"/>
+      <c r="D89" s="55" t="s">
         <v>37</v>
       </c>
-      <c r="E89" s="33"/>
-      <c r="F89" s="34"/>
-      <c r="G89" s="40" t="s">
+      <c r="E89" s="54"/>
+      <c r="F89" s="45"/>
+      <c r="G89" s="55" t="s">
         <v>38</v>
       </c>
-      <c r="H89" s="33"/>
-      <c r="I89" s="34"/>
+      <c r="H89" s="54"/>
+      <c r="I89" s="45"/>
       <c r="J89" s="1"/>
       <c r="K89" s="1"/>
       <c r="L89" s="1"/>
@@ -3652,15 +3647,15 @@
       <c r="Z89" s="1"/>
     </row>
     <row r="90" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A90" s="41"/>
-      <c r="B90" s="38"/>
-      <c r="C90" s="38"/>
-      <c r="D90" s="38"/>
-      <c r="E90" s="38"/>
-      <c r="F90" s="38"/>
-      <c r="G90" s="38"/>
-      <c r="H90" s="38"/>
-      <c r="I90" s="38"/>
+      <c r="A90" s="69"/>
+      <c r="B90" s="67"/>
+      <c r="C90" s="67"/>
+      <c r="D90" s="67"/>
+      <c r="E90" s="67"/>
+      <c r="F90" s="67"/>
+      <c r="G90" s="67"/>
+      <c r="H90" s="67"/>
+      <c r="I90" s="67"/>
       <c r="J90" s="1"/>
       <c r="K90" s="1"/>
       <c r="L90" s="1"/>
@@ -3680,19 +3675,19 @@
       <c r="Z90" s="1"/>
     </row>
     <row r="91" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A91" s="42" t="s">
+      <c r="A91" s="70" t="s">
         <v>39</v>
       </c>
-      <c r="B91" s="43"/>
-      <c r="C91" s="44"/>
-      <c r="D91" s="45"/>
-      <c r="E91" s="38"/>
-      <c r="F91" s="46" t="s">
+      <c r="B91" s="41"/>
+      <c r="C91" s="42"/>
+      <c r="D91" s="71"/>
+      <c r="E91" s="67"/>
+      <c r="F91" s="72" t="s">
         <v>40</v>
       </c>
-      <c r="G91" s="38"/>
-      <c r="H91" s="38"/>
-      <c r="I91" s="47"/>
+      <c r="G91" s="67"/>
+      <c r="H91" s="67"/>
+      <c r="I91" s="73"/>
       <c r="J91" s="1"/>
       <c r="K91" s="1"/>
       <c r="L91" s="1"/>
@@ -3721,16 +3716,16 @@
       <c r="C92" s="3" t="s">
         <v>43</v>
       </c>
-      <c r="D92" s="38"/>
-      <c r="E92" s="38"/>
+      <c r="D92" s="67"/>
+      <c r="E92" s="67"/>
       <c r="F92" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="G92" s="35" t="s">
+      <c r="G92" s="44" t="s">
         <v>44</v>
       </c>
-      <c r="H92" s="33"/>
-      <c r="I92" s="34"/>
+      <c r="H92" s="54"/>
+      <c r="I92" s="45"/>
       <c r="J92" s="1"/>
       <c r="K92" s="1"/>
       <c r="L92" s="1"/>
@@ -3755,12 +3750,12 @@
       </c>
       <c r="B93" s="8"/>
       <c r="C93" s="8"/>
-      <c r="D93" s="38"/>
-      <c r="E93" s="38"/>
+      <c r="D93" s="67"/>
+      <c r="E93" s="67"/>
       <c r="F93" s="4"/>
-      <c r="G93" s="48"/>
-      <c r="H93" s="33"/>
-      <c r="I93" s="34"/>
+      <c r="G93" s="64"/>
+      <c r="H93" s="54"/>
+      <c r="I93" s="45"/>
       <c r="J93" s="1"/>
       <c r="K93" s="1"/>
       <c r="L93" s="1"/>
@@ -3785,12 +3780,12 @@
       </c>
       <c r="B94" s="8"/>
       <c r="C94" s="8"/>
-      <c r="D94" s="38"/>
-      <c r="E94" s="38"/>
+      <c r="D94" s="67"/>
+      <c r="E94" s="67"/>
       <c r="F94" s="4"/>
-      <c r="G94" s="48"/>
-      <c r="H94" s="33"/>
-      <c r="I94" s="34"/>
+      <c r="G94" s="64"/>
+      <c r="H94" s="54"/>
+      <c r="I94" s="45"/>
       <c r="J94" s="1"/>
       <c r="K94" s="1"/>
       <c r="L94" s="1"/>
@@ -3815,12 +3810,12 @@
       </c>
       <c r="B95" s="8"/>
       <c r="C95" s="8"/>
-      <c r="D95" s="38"/>
-      <c r="E95" s="38"/>
+      <c r="D95" s="67"/>
+      <c r="E95" s="67"/>
       <c r="F95" s="4"/>
-      <c r="G95" s="48"/>
-      <c r="H95" s="33"/>
-      <c r="I95" s="34"/>
+      <c r="G95" s="64"/>
+      <c r="H95" s="54"/>
+      <c r="I95" s="45"/>
       <c r="J95" s="1"/>
       <c r="K95" s="1"/>
       <c r="L95" s="1"/>
@@ -3845,12 +3840,12 @@
       </c>
       <c r="B96" s="8"/>
       <c r="C96" s="8"/>
-      <c r="D96" s="38"/>
-      <c r="E96" s="38"/>
+      <c r="D96" s="67"/>
+      <c r="E96" s="67"/>
       <c r="F96" s="4"/>
-      <c r="G96" s="48"/>
-      <c r="H96" s="33"/>
-      <c r="I96" s="34"/>
+      <c r="G96" s="64"/>
+      <c r="H96" s="54"/>
+      <c r="I96" s="45"/>
       <c r="J96" s="1"/>
       <c r="K96" s="1"/>
       <c r="L96" s="1"/>
@@ -3875,12 +3870,12 @@
       </c>
       <c r="B97" s="8"/>
       <c r="C97" s="8"/>
-      <c r="D97" s="38"/>
-      <c r="E97" s="38"/>
+      <c r="D97" s="67"/>
+      <c r="E97" s="67"/>
       <c r="F97" s="4"/>
-      <c r="G97" s="48"/>
-      <c r="H97" s="33"/>
-      <c r="I97" s="34"/>
+      <c r="G97" s="64"/>
+      <c r="H97" s="54"/>
+      <c r="I97" s="45"/>
       <c r="J97" s="1"/>
       <c r="K97" s="1"/>
       <c r="L97" s="1"/>
@@ -3905,12 +3900,12 @@
       </c>
       <c r="B98" s="8"/>
       <c r="C98" s="8"/>
-      <c r="D98" s="38"/>
-      <c r="E98" s="38"/>
+      <c r="D98" s="67"/>
+      <c r="E98" s="67"/>
       <c r="F98" s="4"/>
-      <c r="G98" s="48"/>
-      <c r="H98" s="33"/>
-      <c r="I98" s="34"/>
+      <c r="G98" s="64"/>
+      <c r="H98" s="54"/>
+      <c r="I98" s="45"/>
       <c r="J98" s="1"/>
       <c r="K98" s="1"/>
       <c r="L98" s="1"/>
@@ -3935,12 +3930,12 @@
       </c>
       <c r="B99" s="8"/>
       <c r="C99" s="8"/>
-      <c r="D99" s="38"/>
-      <c r="E99" s="38"/>
+      <c r="D99" s="67"/>
+      <c r="E99" s="67"/>
       <c r="F99" s="4"/>
-      <c r="G99" s="48"/>
-      <c r="H99" s="33"/>
-      <c r="I99" s="34"/>
+      <c r="G99" s="64"/>
+      <c r="H99" s="54"/>
+      <c r="I99" s="45"/>
       <c r="J99" s="1"/>
       <c r="K99" s="1"/>
       <c r="L99" s="1"/>
@@ -3963,14 +3958,14 @@
       <c r="A100" s="3" t="s">
         <v>52</v>
       </c>
-      <c r="B100" s="36"/>
-      <c r="C100" s="34"/>
-      <c r="D100" s="37"/>
-      <c r="E100" s="37"/>
-      <c r="F100" s="38"/>
-      <c r="G100" s="38"/>
-      <c r="H100" s="38"/>
-      <c r="I100" s="38"/>
+      <c r="B100" s="76"/>
+      <c r="C100" s="45"/>
+      <c r="D100" s="66"/>
+      <c r="E100" s="66"/>
+      <c r="F100" s="67"/>
+      <c r="G100" s="67"/>
+      <c r="H100" s="67"/>
+      <c r="I100" s="67"/>
       <c r="J100" s="1"/>
       <c r="K100" s="1"/>
       <c r="L100" s="1"/>
@@ -3990,15 +3985,15 @@
       <c r="Z100" s="1"/>
     </row>
     <row r="101" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A101" s="37"/>
-      <c r="B101" s="38"/>
-      <c r="C101" s="38"/>
-      <c r="D101" s="38"/>
-      <c r="E101" s="38"/>
-      <c r="F101" s="38"/>
-      <c r="G101" s="38"/>
-      <c r="H101" s="38"/>
-      <c r="I101" s="38"/>
+      <c r="A101" s="66"/>
+      <c r="B101" s="67"/>
+      <c r="C101" s="67"/>
+      <c r="D101" s="67"/>
+      <c r="E101" s="67"/>
+      <c r="F101" s="67"/>
+      <c r="G101" s="67"/>
+      <c r="H101" s="67"/>
+      <c r="I101" s="67"/>
       <c r="J101" s="1"/>
       <c r="K101" s="1"/>
       <c r="L101" s="1"/>
@@ -4018,17 +4013,17 @@
       <c r="Z101" s="1"/>
     </row>
     <row r="102" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A102" s="39" t="s">
+      <c r="A102" s="68" t="s">
         <v>53</v>
       </c>
-      <c r="B102" s="29"/>
-      <c r="C102" s="29"/>
-      <c r="D102" s="29"/>
-      <c r="E102" s="29"/>
-      <c r="F102" s="29"/>
-      <c r="G102" s="29"/>
-      <c r="H102" s="29"/>
-      <c r="I102" s="30"/>
+      <c r="B102" s="28"/>
+      <c r="C102" s="28"/>
+      <c r="D102" s="28"/>
+      <c r="E102" s="28"/>
+      <c r="F102" s="28"/>
+      <c r="G102" s="28"/>
+      <c r="H102" s="28"/>
+      <c r="I102" s="29"/>
       <c r="J102" s="1"/>
       <c r="K102" s="1"/>
       <c r="L102" s="1"/>
@@ -4051,14 +4046,14 @@
       <c r="A103" s="3" t="s">
         <v>54</v>
       </c>
-      <c r="B103" s="35" t="s">
+      <c r="B103" s="44" t="s">
         <v>55</v>
       </c>
-      <c r="C103" s="33"/>
-      <c r="D103" s="33"/>
-      <c r="E103" s="33"/>
-      <c r="F103" s="33"/>
-      <c r="G103" s="33"/>
+      <c r="C103" s="54"/>
+      <c r="D103" s="54"/>
+      <c r="E103" s="54"/>
+      <c r="F103" s="54"/>
+      <c r="G103" s="54"/>
       <c r="H103" s="3" t="s">
         <v>56</v>
       </c>
@@ -4087,14 +4082,14 @@
       <c r="A104" s="9">
         <v>1</v>
       </c>
-      <c r="B104" s="32" t="s">
+      <c r="B104" s="74" t="s">
         <v>58</v>
       </c>
-      <c r="C104" s="33"/>
-      <c r="D104" s="33"/>
-      <c r="E104" s="33"/>
-      <c r="F104" s="33"/>
-      <c r="G104" s="34"/>
+      <c r="C104" s="54"/>
+      <c r="D104" s="54"/>
+      <c r="E104" s="54"/>
+      <c r="F104" s="54"/>
+      <c r="G104" s="45"/>
       <c r="H104" s="4"/>
       <c r="I104" s="4"/>
       <c r="J104" s="1"/>
@@ -4119,14 +4114,14 @@
       <c r="A105" s="9">
         <v>2</v>
       </c>
-      <c r="B105" s="32" t="s">
+      <c r="B105" s="74" t="s">
         <v>59</v>
       </c>
-      <c r="C105" s="33"/>
-      <c r="D105" s="33"/>
-      <c r="E105" s="33"/>
-      <c r="F105" s="33"/>
-      <c r="G105" s="34"/>
+      <c r="C105" s="54"/>
+      <c r="D105" s="54"/>
+      <c r="E105" s="54"/>
+      <c r="F105" s="54"/>
+      <c r="G105" s="45"/>
       <c r="H105" s="4"/>
       <c r="I105" s="4"/>
       <c r="J105" s="1"/>
@@ -4151,14 +4146,14 @@
       <c r="A106" s="9">
         <v>3</v>
       </c>
-      <c r="B106" s="32" t="s">
+      <c r="B106" s="74" t="s">
         <v>60</v>
       </c>
-      <c r="C106" s="33"/>
-      <c r="D106" s="33"/>
-      <c r="E106" s="33"/>
-      <c r="F106" s="33"/>
-      <c r="G106" s="34"/>
+      <c r="C106" s="54"/>
+      <c r="D106" s="54"/>
+      <c r="E106" s="54"/>
+      <c r="F106" s="54"/>
+      <c r="G106" s="45"/>
       <c r="H106" s="4"/>
       <c r="I106" s="4"/>
       <c r="J106" s="1"/>
@@ -4183,14 +4178,14 @@
       <c r="A107" s="9">
         <v>4</v>
       </c>
-      <c r="B107" s="32" t="s">
+      <c r="B107" s="74" t="s">
         <v>61</v>
       </c>
-      <c r="C107" s="33"/>
-      <c r="D107" s="33"/>
-      <c r="E107" s="33"/>
-      <c r="F107" s="33"/>
-      <c r="G107" s="34"/>
+      <c r="C107" s="54"/>
+      <c r="D107" s="54"/>
+      <c r="E107" s="54"/>
+      <c r="F107" s="54"/>
+      <c r="G107" s="45"/>
       <c r="H107" s="4"/>
       <c r="I107" s="4"/>
       <c r="J107" s="1"/>
@@ -4215,14 +4210,14 @@
       <c r="A108" s="9">
         <v>5</v>
       </c>
-      <c r="B108" s="32" t="s">
+      <c r="B108" s="74" t="s">
         <v>62</v>
       </c>
-      <c r="C108" s="33"/>
-      <c r="D108" s="33"/>
-      <c r="E108" s="33"/>
-      <c r="F108" s="33"/>
-      <c r="G108" s="34"/>
+      <c r="C108" s="54"/>
+      <c r="D108" s="54"/>
+      <c r="E108" s="54"/>
+      <c r="F108" s="54"/>
+      <c r="G108" s="45"/>
       <c r="H108" s="4"/>
       <c r="I108" s="4"/>
       <c r="J108" s="1"/>
@@ -4247,14 +4242,14 @@
       <c r="A109" s="9">
         <v>6</v>
       </c>
-      <c r="B109" s="32" t="s">
+      <c r="B109" s="74" t="s">
         <v>63</v>
       </c>
-      <c r="C109" s="33"/>
-      <c r="D109" s="33"/>
-      <c r="E109" s="33"/>
-      <c r="F109" s="33"/>
-      <c r="G109" s="34"/>
+      <c r="C109" s="54"/>
+      <c r="D109" s="54"/>
+      <c r="E109" s="54"/>
+      <c r="F109" s="54"/>
+      <c r="G109" s="45"/>
       <c r="H109" s="4"/>
       <c r="I109" s="4"/>
       <c r="J109" s="1"/>
@@ -4279,14 +4274,14 @@
       <c r="A110" s="9">
         <v>7</v>
       </c>
-      <c r="B110" s="32" t="s">
+      <c r="B110" s="74" t="s">
         <v>64</v>
       </c>
-      <c r="C110" s="33"/>
-      <c r="D110" s="33"/>
-      <c r="E110" s="33"/>
-      <c r="F110" s="33"/>
-      <c r="G110" s="34"/>
+      <c r="C110" s="54"/>
+      <c r="D110" s="54"/>
+      <c r="E110" s="54"/>
+      <c r="F110" s="54"/>
+      <c r="G110" s="45"/>
       <c r="H110" s="4"/>
       <c r="I110" s="4"/>
       <c r="J110" s="1"/>
@@ -4311,14 +4306,14 @@
       <c r="A111" s="9">
         <v>8</v>
       </c>
-      <c r="B111" s="32" t="s">
+      <c r="B111" s="74" t="s">
         <v>65</v>
       </c>
-      <c r="C111" s="33"/>
-      <c r="D111" s="33"/>
-      <c r="E111" s="33"/>
-      <c r="F111" s="33"/>
-      <c r="G111" s="34"/>
+      <c r="C111" s="54"/>
+      <c r="D111" s="54"/>
+      <c r="E111" s="54"/>
+      <c r="F111" s="54"/>
+      <c r="G111" s="45"/>
       <c r="H111" s="4"/>
       <c r="I111" s="4"/>
       <c r="J111" s="1"/>
@@ -4343,14 +4338,14 @@
       <c r="A112" s="9">
         <v>9</v>
       </c>
-      <c r="B112" s="32" t="s">
+      <c r="B112" s="74" t="s">
         <v>66</v>
       </c>
-      <c r="C112" s="33"/>
-      <c r="D112" s="33"/>
-      <c r="E112" s="33"/>
-      <c r="F112" s="33"/>
-      <c r="G112" s="34"/>
+      <c r="C112" s="54"/>
+      <c r="D112" s="54"/>
+      <c r="E112" s="54"/>
+      <c r="F112" s="54"/>
+      <c r="G112" s="45"/>
       <c r="H112" s="4"/>
       <c r="I112" s="4"/>
       <c r="J112" s="1"/>
@@ -4375,14 +4370,14 @@
       <c r="A113" s="9">
         <v>10</v>
       </c>
-      <c r="B113" s="32" t="s">
+      <c r="B113" s="74" t="s">
         <v>67</v>
       </c>
-      <c r="C113" s="33"/>
-      <c r="D113" s="33"/>
-      <c r="E113" s="33"/>
-      <c r="F113" s="33"/>
-      <c r="G113" s="34"/>
+      <c r="C113" s="54"/>
+      <c r="D113" s="54"/>
+      <c r="E113" s="54"/>
+      <c r="F113" s="54"/>
+      <c r="G113" s="45"/>
       <c r="H113" s="4"/>
       <c r="I113" s="4"/>
       <c r="J113" s="1"/>
@@ -4407,14 +4402,14 @@
       <c r="A114" s="9">
         <v>11</v>
       </c>
-      <c r="B114" s="32" t="s">
+      <c r="B114" s="74" t="s">
         <v>68</v>
       </c>
-      <c r="C114" s="33"/>
-      <c r="D114" s="33"/>
-      <c r="E114" s="33"/>
-      <c r="F114" s="33"/>
-      <c r="G114" s="34"/>
+      <c r="C114" s="54"/>
+      <c r="D114" s="54"/>
+      <c r="E114" s="54"/>
+      <c r="F114" s="54"/>
+      <c r="G114" s="45"/>
       <c r="H114" s="4"/>
       <c r="I114" s="4"/>
       <c r="J114" s="1"/>
@@ -4439,14 +4434,14 @@
       <c r="A115" s="9">
         <v>12</v>
       </c>
-      <c r="B115" s="32" t="s">
+      <c r="B115" s="74" t="s">
         <v>69</v>
       </c>
-      <c r="C115" s="33"/>
-      <c r="D115" s="33"/>
-      <c r="E115" s="33"/>
-      <c r="F115" s="33"/>
-      <c r="G115" s="34"/>
+      <c r="C115" s="54"/>
+      <c r="D115" s="54"/>
+      <c r="E115" s="54"/>
+      <c r="F115" s="54"/>
+      <c r="G115" s="45"/>
       <c r="H115" s="4"/>
       <c r="I115" s="4"/>
       <c r="J115" s="1"/>
@@ -4468,17 +4463,17 @@
       <c r="Z115" s="1"/>
     </row>
     <row r="116" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A116" s="31" t="s">
+      <c r="A116" s="56" t="s">
         <v>52</v>
       </c>
-      <c r="B116" s="29"/>
-      <c r="C116" s="29"/>
-      <c r="D116" s="29"/>
-      <c r="E116" s="29"/>
-      <c r="F116" s="29"/>
-      <c r="G116" s="29"/>
-      <c r="H116" s="29"/>
-      <c r="I116" s="30"/>
+      <c r="B116" s="28"/>
+      <c r="C116" s="28"/>
+      <c r="D116" s="28"/>
+      <c r="E116" s="28"/>
+      <c r="F116" s="28"/>
+      <c r="G116" s="28"/>
+      <c r="H116" s="28"/>
+      <c r="I116" s="29"/>
       <c r="J116" s="1"/>
       <c r="K116" s="1"/>
       <c r="L116" s="1"/>
@@ -4498,15 +4493,15 @@
       <c r="Z116" s="1"/>
     </row>
     <row r="117" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A117" s="28"/>
-      <c r="B117" s="29"/>
-      <c r="C117" s="29"/>
-      <c r="D117" s="29"/>
-      <c r="E117" s="29"/>
-      <c r="F117" s="29"/>
-      <c r="G117" s="29"/>
-      <c r="H117" s="29"/>
-      <c r="I117" s="30"/>
+      <c r="A117" s="27"/>
+      <c r="B117" s="28"/>
+      <c r="C117" s="28"/>
+      <c r="D117" s="28"/>
+      <c r="E117" s="28"/>
+      <c r="F117" s="28"/>
+      <c r="G117" s="28"/>
+      <c r="H117" s="28"/>
+      <c r="I117" s="29"/>
       <c r="J117" s="1"/>
       <c r="K117" s="1"/>
       <c r="L117" s="1"/>
@@ -4526,15 +4521,15 @@
       <c r="Z117" s="1"/>
     </row>
     <row r="118" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A118" s="28"/>
-      <c r="B118" s="29"/>
-      <c r="C118" s="29"/>
-      <c r="D118" s="29"/>
-      <c r="E118" s="29"/>
-      <c r="F118" s="29"/>
-      <c r="G118" s="29"/>
-      <c r="H118" s="29"/>
-      <c r="I118" s="30"/>
+      <c r="A118" s="27"/>
+      <c r="B118" s="28"/>
+      <c r="C118" s="28"/>
+      <c r="D118" s="28"/>
+      <c r="E118" s="28"/>
+      <c r="F118" s="28"/>
+      <c r="G118" s="28"/>
+      <c r="H118" s="28"/>
+      <c r="I118" s="29"/>
       <c r="J118" s="1"/>
       <c r="K118" s="1"/>
       <c r="L118" s="1"/>
@@ -4554,15 +4549,15 @@
       <c r="Z118" s="1"/>
     </row>
     <row r="119" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A119" s="28"/>
-      <c r="B119" s="29"/>
-      <c r="C119" s="29"/>
-      <c r="D119" s="29"/>
-      <c r="E119" s="29"/>
-      <c r="F119" s="29"/>
-      <c r="G119" s="29"/>
-      <c r="H119" s="29"/>
-      <c r="I119" s="30"/>
+      <c r="A119" s="27"/>
+      <c r="B119" s="28"/>
+      <c r="C119" s="28"/>
+      <c r="D119" s="28"/>
+      <c r="E119" s="28"/>
+      <c r="F119" s="28"/>
+      <c r="G119" s="28"/>
+      <c r="H119" s="28"/>
+      <c r="I119" s="29"/>
       <c r="J119" s="1"/>
       <c r="K119" s="1"/>
       <c r="L119" s="1"/>
@@ -4582,15 +4577,15 @@
       <c r="Z119" s="1"/>
     </row>
     <row r="120" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A120" s="28"/>
-      <c r="B120" s="29"/>
-      <c r="C120" s="29"/>
-      <c r="D120" s="29"/>
-      <c r="E120" s="29"/>
-      <c r="F120" s="29"/>
-      <c r="G120" s="29"/>
-      <c r="H120" s="29"/>
-      <c r="I120" s="30"/>
+      <c r="A120" s="27"/>
+      <c r="B120" s="28"/>
+      <c r="C120" s="28"/>
+      <c r="D120" s="28"/>
+      <c r="E120" s="28"/>
+      <c r="F120" s="28"/>
+      <c r="G120" s="28"/>
+      <c r="H120" s="28"/>
+      <c r="I120" s="29"/>
       <c r="J120" s="1"/>
       <c r="K120" s="1"/>
       <c r="L120" s="1"/>
@@ -4610,15 +4605,15 @@
       <c r="Z120" s="1"/>
     </row>
     <row r="121" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A121" s="28"/>
-      <c r="B121" s="29"/>
-      <c r="C121" s="29"/>
-      <c r="D121" s="29"/>
-      <c r="E121" s="29"/>
-      <c r="F121" s="29"/>
-      <c r="G121" s="29"/>
-      <c r="H121" s="29"/>
-      <c r="I121" s="30"/>
+      <c r="A121" s="27"/>
+      <c r="B121" s="28"/>
+      <c r="C121" s="28"/>
+      <c r="D121" s="28"/>
+      <c r="E121" s="28"/>
+      <c r="F121" s="28"/>
+      <c r="G121" s="28"/>
+      <c r="H121" s="28"/>
+      <c r="I121" s="29"/>
       <c r="J121" s="1"/>
       <c r="K121" s="1"/>
       <c r="L121" s="1"/>
@@ -4638,17 +4633,17 @@
       <c r="Z121" s="1"/>
     </row>
     <row r="122" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A122" s="31" t="s">
+      <c r="A122" s="56" t="s">
         <v>70</v>
       </c>
-      <c r="B122" s="29"/>
-      <c r="C122" s="29"/>
-      <c r="D122" s="29"/>
-      <c r="E122" s="29"/>
-      <c r="F122" s="29"/>
-      <c r="G122" s="29"/>
-      <c r="H122" s="29"/>
-      <c r="I122" s="30"/>
+      <c r="B122" s="28"/>
+      <c r="C122" s="28"/>
+      <c r="D122" s="28"/>
+      <c r="E122" s="28"/>
+      <c r="F122" s="28"/>
+      <c r="G122" s="28"/>
+      <c r="H122" s="28"/>
+      <c r="I122" s="29"/>
       <c r="J122" s="1"/>
       <c r="K122" s="1"/>
       <c r="L122" s="1"/>
@@ -4668,15 +4663,15 @@
       <c r="Z122" s="1"/>
     </row>
     <row r="123" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A123" s="28"/>
-      <c r="B123" s="29"/>
-      <c r="C123" s="29"/>
-      <c r="D123" s="29"/>
-      <c r="E123" s="29"/>
-      <c r="F123" s="29"/>
-      <c r="G123" s="29"/>
-      <c r="H123" s="29"/>
-      <c r="I123" s="30"/>
+      <c r="A123" s="27"/>
+      <c r="B123" s="28"/>
+      <c r="C123" s="28"/>
+      <c r="D123" s="28"/>
+      <c r="E123" s="28"/>
+      <c r="F123" s="28"/>
+      <c r="G123" s="28"/>
+      <c r="H123" s="28"/>
+      <c r="I123" s="29"/>
       <c r="J123" s="1"/>
       <c r="K123" s="1"/>
       <c r="L123" s="1"/>
@@ -4696,15 +4691,15 @@
       <c r="Z123" s="1"/>
     </row>
     <row r="124" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A124" s="28"/>
-      <c r="B124" s="29"/>
-      <c r="C124" s="29"/>
-      <c r="D124" s="29"/>
-      <c r="E124" s="29"/>
-      <c r="F124" s="29"/>
-      <c r="G124" s="29"/>
-      <c r="H124" s="29"/>
-      <c r="I124" s="30"/>
+      <c r="A124" s="27"/>
+      <c r="B124" s="28"/>
+      <c r="C124" s="28"/>
+      <c r="D124" s="28"/>
+      <c r="E124" s="28"/>
+      <c r="F124" s="28"/>
+      <c r="G124" s="28"/>
+      <c r="H124" s="28"/>
+      <c r="I124" s="29"/>
       <c r="J124" s="1"/>
       <c r="K124" s="1"/>
       <c r="L124" s="1"/>
@@ -4724,15 +4719,15 @@
       <c r="Z124" s="1"/>
     </row>
     <row r="125" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A125" s="28"/>
-      <c r="B125" s="29"/>
-      <c r="C125" s="29"/>
-      <c r="D125" s="29"/>
-      <c r="E125" s="29"/>
-      <c r="F125" s="29"/>
-      <c r="G125" s="29"/>
-      <c r="H125" s="29"/>
-      <c r="I125" s="30"/>
+      <c r="A125" s="27"/>
+      <c r="B125" s="28"/>
+      <c r="C125" s="28"/>
+      <c r="D125" s="28"/>
+      <c r="E125" s="28"/>
+      <c r="F125" s="28"/>
+      <c r="G125" s="28"/>
+      <c r="H125" s="28"/>
+      <c r="I125" s="29"/>
       <c r="J125" s="1"/>
       <c r="K125" s="1"/>
       <c r="L125" s="1"/>
@@ -4752,15 +4747,15 @@
       <c r="Z125" s="1"/>
     </row>
     <row r="126" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A126" s="28"/>
-      <c r="B126" s="29"/>
-      <c r="C126" s="29"/>
-      <c r="D126" s="29"/>
-      <c r="E126" s="29"/>
-      <c r="F126" s="29"/>
-      <c r="G126" s="29"/>
-      <c r="H126" s="29"/>
-      <c r="I126" s="30"/>
+      <c r="A126" s="27"/>
+      <c r="B126" s="28"/>
+      <c r="C126" s="28"/>
+      <c r="D126" s="28"/>
+      <c r="E126" s="28"/>
+      <c r="F126" s="28"/>
+      <c r="G126" s="28"/>
+      <c r="H126" s="28"/>
+      <c r="I126" s="29"/>
       <c r="J126" s="1"/>
       <c r="K126" s="1"/>
       <c r="L126" s="1"/>
@@ -4780,15 +4775,15 @@
       <c r="Z126" s="1"/>
     </row>
     <row r="127" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A127" s="28"/>
-      <c r="B127" s="29"/>
-      <c r="C127" s="29"/>
-      <c r="D127" s="29"/>
-      <c r="E127" s="29"/>
-      <c r="F127" s="29"/>
-      <c r="G127" s="29"/>
-      <c r="H127" s="29"/>
-      <c r="I127" s="30"/>
+      <c r="A127" s="27"/>
+      <c r="B127" s="28"/>
+      <c r="C127" s="28"/>
+      <c r="D127" s="28"/>
+      <c r="E127" s="28"/>
+      <c r="F127" s="28"/>
+      <c r="G127" s="28"/>
+      <c r="H127" s="28"/>
+      <c r="I127" s="29"/>
       <c r="J127" s="1"/>
       <c r="K127" s="1"/>
       <c r="L127" s="1"/>
@@ -4808,17 +4803,17 @@
       <c r="Z127" s="1"/>
     </row>
     <row r="128" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A128" s="31" t="s">
+      <c r="A128" s="56" t="s">
         <v>71</v>
       </c>
-      <c r="B128" s="29"/>
-      <c r="C128" s="29"/>
-      <c r="D128" s="29"/>
-      <c r="E128" s="29"/>
-      <c r="F128" s="29"/>
-      <c r="G128" s="29"/>
-      <c r="H128" s="29"/>
-      <c r="I128" s="30"/>
+      <c r="B128" s="28"/>
+      <c r="C128" s="28"/>
+      <c r="D128" s="28"/>
+      <c r="E128" s="28"/>
+      <c r="F128" s="28"/>
+      <c r="G128" s="28"/>
+      <c r="H128" s="28"/>
+      <c r="I128" s="29"/>
       <c r="J128" s="1"/>
       <c r="K128" s="1"/>
       <c r="L128" s="1"/>
@@ -4838,15 +4833,15 @@
       <c r="Z128" s="1"/>
     </row>
     <row r="129" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A129" s="28"/>
-      <c r="B129" s="29"/>
-      <c r="C129" s="29"/>
-      <c r="D129" s="29"/>
-      <c r="E129" s="29"/>
-      <c r="F129" s="29"/>
-      <c r="G129" s="29"/>
-      <c r="H129" s="29"/>
-      <c r="I129" s="30"/>
+      <c r="A129" s="27"/>
+      <c r="B129" s="28"/>
+      <c r="C129" s="28"/>
+      <c r="D129" s="28"/>
+      <c r="E129" s="28"/>
+      <c r="F129" s="28"/>
+      <c r="G129" s="28"/>
+      <c r="H129" s="28"/>
+      <c r="I129" s="29"/>
       <c r="J129" s="1"/>
       <c r="K129" s="1"/>
       <c r="L129" s="1"/>
@@ -4866,15 +4861,15 @@
       <c r="Z129" s="1"/>
     </row>
     <row r="130" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A130" s="28"/>
-      <c r="B130" s="29"/>
-      <c r="C130" s="29"/>
-      <c r="D130" s="29"/>
-      <c r="E130" s="29"/>
-      <c r="F130" s="29"/>
-      <c r="G130" s="29"/>
-      <c r="H130" s="29"/>
-      <c r="I130" s="30"/>
+      <c r="A130" s="27"/>
+      <c r="B130" s="28"/>
+      <c r="C130" s="28"/>
+      <c r="D130" s="28"/>
+      <c r="E130" s="28"/>
+      <c r="F130" s="28"/>
+      <c r="G130" s="28"/>
+      <c r="H130" s="28"/>
+      <c r="I130" s="29"/>
       <c r="J130" s="1"/>
       <c r="K130" s="1"/>
       <c r="L130" s="1"/>
@@ -4894,15 +4889,15 @@
       <c r="Z130" s="1"/>
     </row>
     <row r="131" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A131" s="28"/>
-      <c r="B131" s="29"/>
-      <c r="C131" s="29"/>
-      <c r="D131" s="29"/>
-      <c r="E131" s="29"/>
-      <c r="F131" s="29"/>
-      <c r="G131" s="29"/>
-      <c r="H131" s="29"/>
-      <c r="I131" s="30"/>
+      <c r="A131" s="27"/>
+      <c r="B131" s="28"/>
+      <c r="C131" s="28"/>
+      <c r="D131" s="28"/>
+      <c r="E131" s="28"/>
+      <c r="F131" s="28"/>
+      <c r="G131" s="28"/>
+      <c r="H131" s="28"/>
+      <c r="I131" s="29"/>
       <c r="J131" s="1"/>
       <c r="K131" s="1"/>
       <c r="L131" s="1"/>
@@ -4922,15 +4917,15 @@
       <c r="Z131" s="1"/>
     </row>
     <row r="132" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A132" s="28"/>
-      <c r="B132" s="29"/>
-      <c r="C132" s="29"/>
-      <c r="D132" s="29"/>
-      <c r="E132" s="29"/>
-      <c r="F132" s="29"/>
-      <c r="G132" s="29"/>
-      <c r="H132" s="29"/>
-      <c r="I132" s="30"/>
+      <c r="A132" s="27"/>
+      <c r="B132" s="28"/>
+      <c r="C132" s="28"/>
+      <c r="D132" s="28"/>
+      <c r="E132" s="28"/>
+      <c r="F132" s="28"/>
+      <c r="G132" s="28"/>
+      <c r="H132" s="28"/>
+      <c r="I132" s="29"/>
       <c r="J132" s="1"/>
       <c r="K132" s="1"/>
       <c r="L132" s="1"/>
@@ -4950,15 +4945,15 @@
       <c r="Z132" s="1"/>
     </row>
     <row r="133" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A133" s="77"/>
-      <c r="B133" s="78"/>
-      <c r="C133" s="78"/>
-      <c r="D133" s="78"/>
-      <c r="E133" s="78"/>
-      <c r="F133" s="78"/>
-      <c r="G133" s="78"/>
-      <c r="H133" s="78"/>
-      <c r="I133" s="79"/>
+      <c r="A133" s="30"/>
+      <c r="B133" s="31"/>
+      <c r="C133" s="31"/>
+      <c r="D133" s="31"/>
+      <c r="E133" s="31"/>
+      <c r="F133" s="31"/>
+      <c r="G133" s="31"/>
+      <c r="H133" s="31"/>
+      <c r="I133" s="32"/>
       <c r="J133" s="1"/>
       <c r="K133" s="1"/>
       <c r="L133" s="1"/>
@@ -11027,39 +11022,38 @@
     </row>
   </sheetData>
   <mergeCells count="81">
-    <mergeCell ref="A132:I132"/>
-    <mergeCell ref="A133:I133"/>
-    <mergeCell ref="A8:B8"/>
-    <mergeCell ref="A9:B9"/>
-    <mergeCell ref="C8:C9"/>
-    <mergeCell ref="A1:I2"/>
-    <mergeCell ref="A3:I3"/>
-    <mergeCell ref="A4:I4"/>
-    <mergeCell ref="E6:F6"/>
-    <mergeCell ref="E7:F7"/>
-    <mergeCell ref="A5:I5"/>
-    <mergeCell ref="C6:D6"/>
-    <mergeCell ref="C7:D7"/>
-    <mergeCell ref="A6:B6"/>
-    <mergeCell ref="A7:B7"/>
-    <mergeCell ref="A26:I26"/>
-    <mergeCell ref="A47:C47"/>
-    <mergeCell ref="D47:F47"/>
-    <mergeCell ref="G47:I47"/>
-    <mergeCell ref="A10:D10"/>
-    <mergeCell ref="F10:I10"/>
-    <mergeCell ref="E11:E25"/>
-    <mergeCell ref="A24:B24"/>
-    <mergeCell ref="C24:D25"/>
-    <mergeCell ref="F24:G24"/>
-    <mergeCell ref="H24:I25"/>
-    <mergeCell ref="A25:B25"/>
-    <mergeCell ref="F25:G25"/>
-    <mergeCell ref="G98:I98"/>
-    <mergeCell ref="G99:I99"/>
-    <mergeCell ref="A68:C68"/>
-    <mergeCell ref="D68:F68"/>
-    <mergeCell ref="G68:I68"/>
+    <mergeCell ref="B100:C100"/>
+    <mergeCell ref="E100:I101"/>
+    <mergeCell ref="A130:I130"/>
+    <mergeCell ref="A131:I131"/>
+    <mergeCell ref="D8:I9"/>
+    <mergeCell ref="A120:I120"/>
+    <mergeCell ref="A119:I119"/>
+    <mergeCell ref="A118:I118"/>
+    <mergeCell ref="A117:I117"/>
+    <mergeCell ref="B113:G113"/>
+    <mergeCell ref="B114:G114"/>
+    <mergeCell ref="B115:G115"/>
+    <mergeCell ref="A116:I116"/>
+    <mergeCell ref="B103:G103"/>
+    <mergeCell ref="B104:G104"/>
+    <mergeCell ref="B105:G105"/>
+    <mergeCell ref="B106:G106"/>
+    <mergeCell ref="B107:G107"/>
+    <mergeCell ref="A129:I129"/>
+    <mergeCell ref="A122:I122"/>
+    <mergeCell ref="A123:I123"/>
+    <mergeCell ref="A126:I126"/>
+    <mergeCell ref="A127:I127"/>
+    <mergeCell ref="A128:I128"/>
+    <mergeCell ref="A124:I124"/>
+    <mergeCell ref="A125:I125"/>
+    <mergeCell ref="A121:I121"/>
+    <mergeCell ref="B108:G108"/>
+    <mergeCell ref="B109:G109"/>
+    <mergeCell ref="B110:G110"/>
+    <mergeCell ref="B111:G111"/>
+    <mergeCell ref="B112:G112"/>
     <mergeCell ref="A101:C101"/>
     <mergeCell ref="D100:D101"/>
     <mergeCell ref="A102:I102"/>
@@ -11076,38 +11070,39 @@
     <mergeCell ref="G95:I95"/>
     <mergeCell ref="G96:I96"/>
     <mergeCell ref="G97:I97"/>
-    <mergeCell ref="A121:I121"/>
-    <mergeCell ref="B108:G108"/>
-    <mergeCell ref="B109:G109"/>
-    <mergeCell ref="B110:G110"/>
-    <mergeCell ref="B111:G111"/>
-    <mergeCell ref="B112:G112"/>
-    <mergeCell ref="A129:I129"/>
-    <mergeCell ref="A122:I122"/>
-    <mergeCell ref="A123:I123"/>
-    <mergeCell ref="A126:I126"/>
-    <mergeCell ref="A127:I127"/>
-    <mergeCell ref="A128:I128"/>
-    <mergeCell ref="A124:I124"/>
-    <mergeCell ref="A125:I125"/>
-    <mergeCell ref="A130:I130"/>
-    <mergeCell ref="A131:I131"/>
-    <mergeCell ref="D8:I9"/>
-    <mergeCell ref="A120:I120"/>
-    <mergeCell ref="A119:I119"/>
-    <mergeCell ref="A118:I118"/>
-    <mergeCell ref="A117:I117"/>
-    <mergeCell ref="B113:G113"/>
-    <mergeCell ref="B114:G114"/>
-    <mergeCell ref="B115:G115"/>
-    <mergeCell ref="A116:I116"/>
-    <mergeCell ref="B103:G103"/>
-    <mergeCell ref="B104:G104"/>
-    <mergeCell ref="B105:G105"/>
-    <mergeCell ref="B106:G106"/>
-    <mergeCell ref="B107:G107"/>
-    <mergeCell ref="B100:C100"/>
-    <mergeCell ref="E100:I101"/>
+    <mergeCell ref="A25:B25"/>
+    <mergeCell ref="F25:G25"/>
+    <mergeCell ref="G98:I98"/>
+    <mergeCell ref="G99:I99"/>
+    <mergeCell ref="A68:C68"/>
+    <mergeCell ref="D68:F68"/>
+    <mergeCell ref="G68:I68"/>
+    <mergeCell ref="A1:I2"/>
+    <mergeCell ref="A3:I3"/>
+    <mergeCell ref="A4:I4"/>
+    <mergeCell ref="E6:F6"/>
+    <mergeCell ref="E7:F7"/>
+    <mergeCell ref="A5:I5"/>
+    <mergeCell ref="C6:D6"/>
+    <mergeCell ref="C7:D7"/>
+    <mergeCell ref="A6:B6"/>
+    <mergeCell ref="A7:B7"/>
+    <mergeCell ref="A132:I132"/>
+    <mergeCell ref="A133:I133"/>
+    <mergeCell ref="A8:B8"/>
+    <mergeCell ref="A9:B9"/>
+    <mergeCell ref="C8:C9"/>
+    <mergeCell ref="A26:I26"/>
+    <mergeCell ref="A47:C47"/>
+    <mergeCell ref="D47:F47"/>
+    <mergeCell ref="G47:I47"/>
+    <mergeCell ref="A10:D10"/>
+    <mergeCell ref="F10:I10"/>
+    <mergeCell ref="E11:E25"/>
+    <mergeCell ref="A24:B24"/>
+    <mergeCell ref="C24:D25"/>
+    <mergeCell ref="F24:G24"/>
+    <mergeCell ref="H24:I25"/>
   </mergeCells>
   <printOptions horizontalCentered="1" gridLines="1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0" footer="0"/>

</xml_diff>